<commit_message>
Add British Heart Foundation resistance-band video, upgrade Pilates Mat channel
- Add "10 resistance band exercises you can do at home" from British
  Heart Foundation (new approved channel - major UK health charity),
  closing another full-body/long-band exercise target.
- Upgrade "The Girl With The Pilates Mat" from pending to approved
  after deeper review: explicit Master-level certification, 355K
  subscribers, and safety-conscious content for osteoporosis/
  menopause/over-40 audiences.
</commit_message>
<xml_diff>
--- a/YR1/pilates/data/מטריצת_כיסוי_קטלוג_פילאטיס_v5.xlsx
+++ b/YR1/pilates/data/מטריצת_כיסוי_קטלוג_פילאטיס_v5.xlsx
@@ -600,7 +600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:A52"/>
+  <dimension ref="A1:A53"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6171875" defaultRowHeight="13.5" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="115" customWidth="1" style="24" min="1" max="1"/>
@@ -934,16 +934,23 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" t="inlineStr">
+      <c r="A51" s="24" t="inlineStr">
         <is>
           <t>• חיפוש פעיל שביצע Claude (29.08.2026): נוספו 13 סרטונים חדשים (11 תרגילים + 2 שיעורים) שאותרו ואומתו לפי סדר החיפוש המתועד למעלה - בעיקר מערוצי Jessica Valant Pilates, Blogilates ו-Lottie Murphy (מאושרים), ואחד מ-PILATES BY IZZY (ערוץ חדש, נוסף כ'לבדוק ידנית').</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" t="inlineStr">
+      <c r="A52" s="24" t="inlineStr">
         <is>
           <t xml:space="preserve">  תוצאה: 7 מתוך 8 יעדי "חובה" בתרגילים הושלמו/כמעט הושלמו (רק #4 - בטן וליבה+גומיית לולאה+מתחילים - נותר פתוח, לא נמצא סרטון מתאים). 2 יעדי שיעורים נוספים הושלמו.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>• 30.08.2026: נוסף סרטון ספציפי שביקש המשתמש (British Heart Foundation, "10 resistance band exercises you can do at home") - הערוץ נוסף כ"מאושר" (עמותת בריאות לאומית מוכרת). הועלה לגיליון #34 ולמטריצת תרגילים (#28, גוף מלא). שודרג גם ערוץ "The Girl With The Pilates Mat" מ"לבדוק ידנית" ל"מאושר" לאחר בדיקה מעמיקה לבקשת המשתמש - נמצאה הסמכה מפורשת (Master-level Certified Pilates Instructor) וערוץ גדול ומבוסס (355K מנויים) עם התמחות בטיחותית לאוכלוסיות רגישות.</t>
         </is>
       </c>
     </row>
@@ -2522,7 +2529,7 @@
         <v>2</v>
       </c>
       <c r="J30" s="35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K30" s="33">
         <f>IF(J33=0,"חסר",IF(J33&lt;I33,"בתהליך","הושלם"))</f>
@@ -6632,30 +6639,95 @@
       <c r="A35" s="33" t="n">
         <v>34</v>
       </c>
-      <c r="B35" s="36" t="n"/>
-      <c r="C35" s="36" t="n"/>
-      <c r="D35" s="34" t="n"/>
-      <c r="E35" s="33" t="n"/>
-      <c r="F35" s="35" t="n"/>
-      <c r="G35" s="35" t="n"/>
-      <c r="H35" s="33" t="n"/>
-      <c r="I35" s="34" t="n"/>
-      <c r="J35" s="34" t="n"/>
-      <c r="K35" s="34" t="n"/>
-      <c r="L35" s="34" t="n"/>
-      <c r="M35" s="34" t="n"/>
-      <c r="N35" s="35" t="n"/>
-      <c r="O35" s="35" t="n"/>
-      <c r="P35" s="35" t="n"/>
-      <c r="Q35" s="35" t="n"/>
-      <c r="R35" s="35" t="n"/>
-      <c r="S35" s="35" t="n"/>
-      <c r="T35" s="33">
-        <f>IF(COUNT(N37:S37)=0,"",ROUND(AVERAGE(N37:S37),1))</f>
-        <v/>
-      </c>
-      <c r="U35" s="33" t="n"/>
-      <c r="V35" s="36" t="n"/>
+      <c r="B35" s="36" t="inlineStr">
+        <is>
+          <t>10 resistance band exercises you can do at home</t>
+        </is>
+      </c>
+      <c r="C35" s="36" t="inlineStr">
+        <is>
+          <t>British Heart Foundation</t>
+        </is>
+      </c>
+      <c r="D35" s="34" t="inlineStr">
+        <is>
+          <t>British Heart Foundation</t>
+        </is>
+      </c>
+      <c r="E35" s="33" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=fgKHFLe654U</t>
+        </is>
+      </c>
+      <c r="F35" s="35" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G35" s="35" t="n">
+        <v>7</v>
+      </c>
+      <c r="H35" s="33" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I35" s="34" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J35" s="34" t="inlineStr">
+        <is>
+          <t>גומיית רצועה ארוכה</t>
+        </is>
+      </c>
+      <c r="K35" s="34" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L35" s="34" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M35" s="34" t="inlineStr">
+        <is>
+          <t>גוף מלא</t>
+        </is>
+      </c>
+      <c r="N35" s="35" t="n">
+        <v>5</v>
+      </c>
+      <c r="O35" s="35" t="n">
+        <v>4</v>
+      </c>
+      <c r="P35" s="35" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q35" s="35" t="n">
+        <v>4</v>
+      </c>
+      <c r="R35" s="35" t="n">
+        <v>4</v>
+      </c>
+      <c r="S35" s="35" t="n">
+        <v>5</v>
+      </c>
+      <c r="T35" s="33" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="U35" s="33" t="inlineStr">
+        <is>
+          <t>לכלול בקטלוג</t>
+        </is>
+      </c>
+      <c r="V35" s="36" t="inlineStr">
+        <is>
+          <t>10 תרגילי גומיית התנגדות לגוף מלא (כולל תרגיל גב עליון עם משיכה מעל הראש - מתאים ל"גומיית רצועה ארוכה"). מקור אמין במיוחד (עמותת בריאות לב) - תוכן בטיחותי ומותאם לקהל רחב, כולל שיקום. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="13.5" customHeight="1" s="25">
       <c r="A36" s="33" t="n">
@@ -6816,7 +6888,7 @@
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation sqref="D2:D41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
-      <formula1>'ערוצים מאושרים'!$B$2:$B$20</formula1>
+      <formula1>'ערוצים מאושרים'!$B$2:$B$21</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -9313,21 +9385,76 @@
       </c>
     </row>
     <row r="35" ht="13.5" customHeight="1" s="25">
-      <c r="A35" s="33" t="n"/>
-      <c r="B35" s="36" t="n"/>
-      <c r="C35" s="36" t="n"/>
-      <c r="D35" s="34" t="n"/>
-      <c r="E35" s="33" t="n"/>
-      <c r="F35" s="35" t="n"/>
-      <c r="G35" s="33" t="n"/>
-      <c r="H35" s="33" t="n"/>
-      <c r="I35" s="34" t="n"/>
-      <c r="J35" s="34" t="n"/>
-      <c r="K35" s="34" t="n"/>
-      <c r="L35" s="34" t="n"/>
-      <c r="M35" s="34" t="n"/>
-      <c r="N35" s="33" t="n"/>
-      <c r="O35" s="36" t="n"/>
+      <c r="A35" s="33" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="36" t="inlineStr">
+        <is>
+          <t>10 resistance band exercises you can do at home</t>
+        </is>
+      </c>
+      <c r="C35" s="36" t="inlineStr">
+        <is>
+          <t>British Heart Foundation</t>
+        </is>
+      </c>
+      <c r="D35" s="34" t="inlineStr">
+        <is>
+          <t>British Heart Foundation</t>
+        </is>
+      </c>
+      <c r="E35" s="33" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=fgKHFLe654U</t>
+        </is>
+      </c>
+      <c r="F35" s="35" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G35" s="33" t="n">
+        <v>7</v>
+      </c>
+      <c r="H35" s="33" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I35" s="34" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J35" s="34" t="inlineStr">
+        <is>
+          <t>גומיית רצועה ארוכה</t>
+        </is>
+      </c>
+      <c r="K35" s="34" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L35" s="34" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M35" s="34" t="inlineStr">
+        <is>
+          <t>גוף מלא</t>
+        </is>
+      </c>
+      <c r="N35" s="33">
+        <f>'מאגר מועמדים'!T35</f>
+        <v/>
+      </c>
+      <c r="O35" s="36" t="inlineStr">
+        <is>
+          <t>אושר לקטלוג. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="13.5" customHeight="1" s="25">
       <c r="A36" s="33" t="n"/>
@@ -9453,7 +9580,7 @@
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation sqref="D2:D41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
-      <formula1>'ערוצים מאושרים'!$B$2:$B$20</formula1>
+      <formula1>'ערוצים מאושרים'!$B$2:$B$21</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -9863,7 +9990,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:K20"/>
+  <dimension ref="A1:K21"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6171875" defaultRowHeight="13.5" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="6" customWidth="1" style="24" min="1" max="1"/>
@@ -10456,24 +10583,24 @@
       </c>
       <c r="D16" s="24" t="inlineStr">
         <is>
-          <t>לבדוק ידנית</t>
+          <t>מאושר</t>
         </is>
       </c>
       <c r="E16" s="24" t="inlineStr">
         <is>
-          <t>שיעורי פילאטיס מלאים עם גומיית התנגדות, כל הרמות</t>
+          <t>שיעורי פילאטיס עומד (standing) עם גומייה/רינג/משקולות, מותאם לנשים 40+, אוסטאופורוזיס, גיל המעבר</t>
         </is>
       </c>
       <c r="F16" s="24" t="inlineStr">
         <is>
-          <t>לא מאומת</t>
+          <t>מוסמכת פילאטיס ברמת Master (Rachel Lawrence), מחברת ספר פילאטיס</t>
         </is>
       </c>
       <c r="G16" s="24" t="inlineStr"/>
       <c r="H16" s="24" t="inlineStr"/>
       <c r="I16" s="24" t="inlineStr">
         <is>
-          <t>אותר במסגרת בניית קטלוג האתר (yairron.com/YR1/pilates); ערוץ יוטיוב חופשי ופעיל, כמה סרטונים נבחרו. טרם בוצע אימות הסמכה מלא.</t>
+          <t>עודכן ע"י Claude, 30.08.2026 - נבדק לעומק לבקשת המשתמש: 355K מנויים, 1,023 סרטונים, פעילה מ-2016, 37.5M+ צפיות (ערוץ גדול ומבוסס משמעותית ממה שהוערך בתחילה). ביו הערוץ כולל הסמכה מפורשת "Master-level Certified Pilates Instructor" + פרסמה ספר ("The Little Book of Pilates"). תוכן עדכני מציג מיקוד בטיחותי ברור לאוכלוסיות רגישות (Safe for Osteoporosis, Menopause Relief, Women Over 40) - עדות טובה לעקרון "אין הבטחות רפואיות מוגזמות + התאמות לרמות שונות". מכירת ספר/בגדים בביו - לא חוסם תוכן וידאו, שלא כמו Pilates Anytime.</t>
         </is>
       </c>
     </row>
@@ -10622,6 +10749,43 @@
       <c r="I20" s="24" t="inlineStr">
         <is>
           <t>אומת מול YouTube בפועל (29.08.2026): ערוץ חדש יחסית (מ-02/2024) אך צמיחה חריגה - 500K+ מנויים בזכות אתגר 25 הימים הוויראלי. הכשרה כמדריכת פילאטיס מזרן מוסמכת מאומתת ממקורות חיצוניים (vidIQ, Marie Claire). טרם אומת ישירות מול אתר/ביו הערוץ עצמו.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>British Heart Foundation</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/@britishheartfoundation</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>מאושר</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>תוכן פעילות גופנית/גומיות התנגדות לבריאות הלב (לא ערוץ פילאטיס ייעודי)</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>עמותת בריאות לאומית מובילה בבריטניה (לא הסמכת פילאטיס אישית)</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>נוסף ע"י Claude, 30.08.2026 - אותר דרך סרטון ספציפי שביקש המשתמש. 114K מנויים, 1,118 סרטונים - עמותה רפואית מוכרת ומבוססת (לא מדריך/ה עצמאי/ת), רמת אמינות גבוהה מאוד למרות שאינה "ערוץ פילאטיס" במובן הרגיל - תוכן פעילות גופנית/שיקום לב מבוסס-בטיחות.</t>
         </is>
       </c>
     </row>
@@ -11672,7 +11836,7 @@
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation sqref="E2:E14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
-      <formula1>'ערוצים מאושרים'!$B$2:$B$20</formula1>
+      <formula1>'ערוצים מאושרים'!$B$2:$B$21</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Add 12 videos from The Girl With The Pilates Mat, close 4 matrix gaps
Reviewed the channel's catalog (mini-band, long resistance band, ring,
and mini-ball content) and added the videos that fit still-open
exercise-matrix targets. Fully closes 4 targets (core+ring,
back+ring, arms+ring, arms+long-band), advances 3 more, and adds
depth beyond target on full-body+long-band (allowed per instructions).
Also fixed a ring-equipment tag inconsistency in videos.json
("טבעת פילאטיס" vs "רינג פילאטיס") to keep the site's filter
taxonomy from splitting into duplicate categories.
</commit_message>
<xml_diff>
--- a/YR1/pilates/data/מטריצת_כיסוי_קטלוג_פילאטיס_v5.xlsx
+++ b/YR1/pilates/data/מטריצת_כיסוי_קטלוג_פילאטיס_v5.xlsx
@@ -600,7 +600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:A53"/>
+  <dimension ref="A1:A54"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6171875" defaultRowHeight="13.5" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="115" customWidth="1" style="24" min="1" max="1"/>
@@ -948,9 +948,16 @@
       </c>
     </row>
     <row r="53">
-      <c r="A53" t="inlineStr">
+      <c r="A53" s="24" t="inlineStr">
         <is>
           <t>• 30.08.2026: נוסף סרטון ספציפי שביקש המשתמש (British Heart Foundation, "10 resistance band exercises you can do at home") - הערוץ נוסף כ"מאושר" (עמותת בריאות לאומית מוכרת). הועלה לגיליון #34 ולמטריצת תרגילים (#28, גוף מלא). שודרג גם ערוץ "The Girl With The Pilates Mat" מ"לבדוק ידנית" ל"מאושר" לאחר בדיקה מעמיקה לבקשת המשתמש - נמצאה הסמכה מפורשת (Master-level Certified Pilates Instructor) וערוץ גדול ומבוסס (355K מנויים) עם התמחות בטיחותית לאוכלוסיות רגישות.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>• 30.08.2026: עברתי על סרטוני הערוץ "The Girl With The Pilates Mat" לבקשת המשתמש - נוספו 12 סרטונים חדשים (#35-46). סגרו לגמרי: #7,#13,#25,#26 (הושלמו); הרחיבו משמעותית: #4,#24,#28 (חלקי); #29 עבר את היעד בהרבה (מותר לפי הנחיית המשתמש). 2 סרטונים (בינוני/כדור-קטן-בינוני) לא תאמו משבצת קיימת - נוספו כתוכן בונוס.</t>
         </is>
       </c>
     </row>
@@ -1242,7 +1249,7 @@
         <v>2</v>
       </c>
       <c r="J5" s="35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K5" s="33">
         <f>IF(J5=0,"חסר",IF(J5&lt;I5,"בתהליך","הושלם"))</f>
@@ -1395,7 +1402,7 @@
         <v>2</v>
       </c>
       <c r="J8" s="35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K8" s="33">
         <f>IF(J8=0,"חסר",IF(J8&lt;I8,"בתהליך","הושלם"))</f>
@@ -1701,7 +1708,7 @@
         <v>1</v>
       </c>
       <c r="J14" s="35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K14" s="33">
         <f>IF(J14=0,"חסר",IF(J14&lt;I14,"בתהליך","הושלם"))</f>
@@ -2274,7 +2281,7 @@
         <v>2</v>
       </c>
       <c r="J25" s="35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K25" s="33">
         <f>IF(J28=0,"חסר",IF(J28&lt;I28,"בתהליך","הושלם"))</f>
@@ -2325,7 +2332,7 @@
         <v>2</v>
       </c>
       <c r="J26" s="35" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K26" s="33">
         <f>IF(J29=0,"חסר",IF(J29&lt;I29,"בתהליך","הושלם"))</f>
@@ -2376,7 +2383,7 @@
         <v>1</v>
       </c>
       <c r="J27" s="35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K27" s="33">
         <f>IF(J30=0,"חסר",IF(J30&lt;I30,"בתהליך","הושלם"))</f>
@@ -2478,7 +2485,7 @@
         <v>2</v>
       </c>
       <c r="J29" s="35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K29" s="33">
         <f>IF(J32=0,"חסר",IF(J32&lt;I32,"בתהליך","הושלם"))</f>
@@ -2529,7 +2536,7 @@
         <v>2</v>
       </c>
       <c r="J30" s="35" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="K30" s="33">
         <f>IF(J33=0,"חסר",IF(J33&lt;I33,"בתהליך","הושלם"))</f>
@@ -3396,7 +3403,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:V39"/>
+  <dimension ref="A1:V47"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6171875" defaultRowHeight="13.5" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="6" customWidth="1" style="24" min="1" max="1"/>
@@ -6733,120 +6740,1130 @@
       <c r="A36" s="33" t="n">
         <v>35</v>
       </c>
-      <c r="B36" s="36" t="n"/>
-      <c r="C36" s="36" t="n"/>
-      <c r="D36" s="34" t="n"/>
-      <c r="E36" s="33" t="n"/>
-      <c r="F36" s="35" t="n"/>
-      <c r="G36" s="35" t="n"/>
-      <c r="H36" s="33" t="n"/>
-      <c r="I36" s="34" t="n"/>
-      <c r="J36" s="34" t="n"/>
-      <c r="K36" s="34" t="n"/>
-      <c r="L36" s="34" t="n"/>
-      <c r="M36" s="34" t="n"/>
-      <c r="N36" s="35" t="n"/>
-      <c r="O36" s="35" t="n"/>
-      <c r="P36" s="35" t="n"/>
-      <c r="Q36" s="35" t="n"/>
-      <c r="R36" s="35" t="n"/>
-      <c r="S36" s="35" t="n"/>
-      <c r="T36" s="33">
-        <f>IF(COUNT(N38:S38)=0,"",ROUND(AVERAGE(N38:S38),1))</f>
-        <v/>
-      </c>
-      <c r="U36" s="33" t="n"/>
-      <c r="V36" s="36" t="n"/>
+      <c r="B36" s="36" t="inlineStr">
+        <is>
+          <t>Pilates Strength Training with a Mini Band | 15 mins Upper Body | 15 Mins Legs, Core &amp; Glutes</t>
+        </is>
+      </c>
+      <c r="C36" s="36" t="inlineStr">
+        <is>
+          <t>The Girl With The Pilates Mat</t>
+        </is>
+      </c>
+      <c r="D36" s="34" t="inlineStr">
+        <is>
+          <t>The Girl With The Pilates Mat</t>
+        </is>
+      </c>
+      <c r="E36" s="33" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=tD8TW3KmBg4</t>
+        </is>
+      </c>
+      <c r="F36" s="35" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G36" s="35" t="n">
+        <v>56</v>
+      </c>
+      <c r="H36" s="33" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I36" s="34" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J36" s="34" t="inlineStr">
+        <is>
+          <t>גומיית לולאה</t>
+        </is>
+      </c>
+      <c r="K36" s="34" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L36" s="34" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M36" s="34" t="inlineStr">
+        <is>
+          <t>כתפיים וזרועות / ישבן ורגליים / בטן וליבה</t>
+        </is>
+      </c>
+      <c r="N36" s="35" t="n">
+        <v>4</v>
+      </c>
+      <c r="O36" s="35" t="n">
+        <v>4</v>
+      </c>
+      <c r="P36" s="35" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q36" s="35" t="n">
+        <v>5</v>
+      </c>
+      <c r="R36" s="35" t="n">
+        <v>4</v>
+      </c>
+      <c r="S36" s="35" t="n">
+        <v>5</v>
+      </c>
+      <c r="T36" s="33" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="U36" s="33" t="inlineStr">
+        <is>
+          <t>לכלול בקטלוג</t>
+        </is>
+      </c>
+      <c r="V36" s="36" t="inlineStr">
+        <is>
+          <t>ערוץ מאושר (Master-level Certified Pilates Instructor). [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל (oembed+lengthSeconds); לא נצפה תוכן במלואו.]</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="13.5" customHeight="1" s="25">
       <c r="A37" s="33" t="n">
         <v>36</v>
       </c>
-      <c r="B37" s="36" t="n"/>
-      <c r="C37" s="36" t="n"/>
-      <c r="D37" s="34" t="n"/>
-      <c r="E37" s="33" t="n"/>
-      <c r="F37" s="35" t="n"/>
-      <c r="G37" s="35" t="n"/>
-      <c r="H37" s="33" t="n"/>
-      <c r="I37" s="34" t="n"/>
-      <c r="J37" s="34" t="n"/>
-      <c r="K37" s="34" t="n"/>
-      <c r="L37" s="34" t="n"/>
-      <c r="M37" s="34" t="n"/>
-      <c r="N37" s="35" t="n"/>
-      <c r="O37" s="35" t="n"/>
-      <c r="P37" s="35" t="n"/>
-      <c r="Q37" s="35" t="n"/>
-      <c r="R37" s="35" t="n"/>
-      <c r="S37" s="35" t="n"/>
-      <c r="T37" s="33">
-        <f>IF(COUNT(N39:S39)=0,"",ROUND(AVERAGE(N39:S39),1))</f>
-        <v/>
-      </c>
-      <c r="U37" s="33" t="n"/>
-      <c r="V37" s="36" t="n"/>
+      <c r="B37" s="36" t="inlineStr">
+        <is>
+          <t>Pilates Mini Resistance Band Class | 30 Minutes | Full Body Workout</t>
+        </is>
+      </c>
+      <c r="C37" s="36" t="inlineStr">
+        <is>
+          <t>The Girl With The Pilates Mat</t>
+        </is>
+      </c>
+      <c r="D37" s="34" t="inlineStr">
+        <is>
+          <t>The Girl With The Pilates Mat</t>
+        </is>
+      </c>
+      <c r="E37" s="33" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=sh5_uhqLGZw</t>
+        </is>
+      </c>
+      <c r="F37" s="35" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G37" s="35" t="n">
+        <v>48</v>
+      </c>
+      <c r="H37" s="33" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I37" s="34" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J37" s="34" t="inlineStr">
+        <is>
+          <t>גומיית לולאה</t>
+        </is>
+      </c>
+      <c r="K37" s="34" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L37" s="34" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M37" s="34" t="inlineStr">
+        <is>
+          <t>גוף מלא</t>
+        </is>
+      </c>
+      <c r="N37" s="35" t="n">
+        <v>4</v>
+      </c>
+      <c r="O37" s="35" t="n">
+        <v>4</v>
+      </c>
+      <c r="P37" s="35" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q37" s="35" t="n">
+        <v>5</v>
+      </c>
+      <c r="R37" s="35" t="n">
+        <v>4</v>
+      </c>
+      <c r="S37" s="35" t="n">
+        <v>5</v>
+      </c>
+      <c r="T37" s="33" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="U37" s="33" t="inlineStr">
+        <is>
+          <t>לכלול בקטלוג</t>
+        </is>
+      </c>
+      <c r="V37" s="36" t="inlineStr">
+        <is>
+          <t>ערוץ מאושר (Master-level Certified Pilates Instructor). [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל (oembed+lengthSeconds); לא נצפה תוכן במלואו.]</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="13.5" customHeight="1" s="25">
       <c r="A38" s="33" t="n">
         <v>37</v>
       </c>
-      <c r="B38" s="36" t="n"/>
-      <c r="C38" s="36" t="n"/>
-      <c r="D38" s="34" t="n"/>
-      <c r="E38" s="33" t="n"/>
-      <c r="F38" s="35" t="n"/>
-      <c r="G38" s="35" t="n"/>
-      <c r="H38" s="33" t="n"/>
-      <c r="I38" s="34" t="n"/>
-      <c r="J38" s="34" t="n"/>
-      <c r="K38" s="34" t="n"/>
-      <c r="L38" s="34" t="n"/>
-      <c r="M38" s="34" t="n"/>
-      <c r="N38" s="35" t="n"/>
-      <c r="O38" s="35" t="n"/>
-      <c r="P38" s="35" t="n"/>
-      <c r="Q38" s="35" t="n"/>
-      <c r="R38" s="35" t="n"/>
-      <c r="S38" s="35" t="n"/>
-      <c r="T38" s="33">
-        <f>IF(COUNT(N40:S40)=0,"",ROUND(AVERAGE(N40:S40),1))</f>
-        <v/>
-      </c>
-      <c r="U38" s="33" t="n"/>
-      <c r="V38" s="36" t="n"/>
+      <c r="B38" s="36" t="inlineStr">
+        <is>
+          <t>40 MIN FULL BODY MINI BAND WORKOUT | Intermediate Pilates with Mini Band ( Optional)</t>
+        </is>
+      </c>
+      <c r="C38" s="36" t="inlineStr">
+        <is>
+          <t>The Girl With The Pilates Mat</t>
+        </is>
+      </c>
+      <c r="D38" s="34" t="inlineStr">
+        <is>
+          <t>The Girl With The Pilates Mat</t>
+        </is>
+      </c>
+      <c r="E38" s="33" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=F2iru_IAqJ0</t>
+        </is>
+      </c>
+      <c r="F38" s="35" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G38" s="35" t="n">
+        <v>72</v>
+      </c>
+      <c r="H38" s="33" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I38" s="34" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J38" s="34" t="inlineStr">
+        <is>
+          <t>גומיית לולאה</t>
+        </is>
+      </c>
+      <c r="K38" s="34" t="inlineStr">
+        <is>
+          <t>בינוני</t>
+        </is>
+      </c>
+      <c r="L38" s="34" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M38" s="34" t="inlineStr">
+        <is>
+          <t>גוף מלא</t>
+        </is>
+      </c>
+      <c r="N38" s="35" t="n">
+        <v>4</v>
+      </c>
+      <c r="O38" s="35" t="n">
+        <v>4</v>
+      </c>
+      <c r="P38" s="35" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q38" s="35" t="n">
+        <v>5</v>
+      </c>
+      <c r="R38" s="35" t="n">
+        <v>4</v>
+      </c>
+      <c r="S38" s="35" t="n">
+        <v>5</v>
+      </c>
+      <c r="T38" s="33" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="U38" s="33" t="inlineStr">
+        <is>
+          <t>לכלול בקטלוג</t>
+        </is>
+      </c>
+      <c r="V38" s="36" t="inlineStr">
+        <is>
+          <t>ערוץ מאושר (Master-level Certified Pilates Instructor). לא תואם משבצת קיימת (רמת בינוני לגוף מלא לא מוגדרת במטריצה) - תוכן בונוס. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל (oembed+lengthSeconds); לא נצפה תוכן במלואו.]</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="13.5" customHeight="1" s="25">
       <c r="A39" s="33" t="n">
         <v>38</v>
       </c>
-      <c r="B39" s="36" t="n"/>
-      <c r="C39" s="36" t="n"/>
-      <c r="D39" s="34" t="n"/>
-      <c r="E39" s="33" t="n"/>
-      <c r="F39" s="35" t="n"/>
-      <c r="G39" s="35" t="n"/>
-      <c r="H39" s="33" t="n"/>
-      <c r="I39" s="34" t="n"/>
-      <c r="J39" s="34" t="n"/>
-      <c r="K39" s="34" t="n"/>
-      <c r="L39" s="34" t="n"/>
-      <c r="M39" s="34" t="n"/>
-      <c r="N39" s="35" t="n"/>
-      <c r="O39" s="35" t="n"/>
-      <c r="P39" s="35" t="n"/>
-      <c r="Q39" s="35" t="n"/>
-      <c r="R39" s="35" t="n"/>
-      <c r="S39" s="35" t="n"/>
-      <c r="T39" s="33">
-        <f>IF(COUNT(N41:S41)=0,"",ROUND(AVERAGE(N41:S41),1))</f>
-        <v/>
-      </c>
-      <c r="U39" s="33" t="n"/>
-      <c r="V39" s="36" t="n"/>
-    </row>
-    <row r="40" ht="13.5" customHeight="1" s="25"/>
-    <row r="41" ht="13.5" customHeight="1" s="25"/>
+      <c r="B39" s="36" t="inlineStr">
+        <is>
+          <t>Pilates Mini Ball Workout for Core Strength and Stability | Intermediate Level | 30 Min</t>
+        </is>
+      </c>
+      <c r="C39" s="36" t="inlineStr">
+        <is>
+          <t>The Girl With The Pilates Mat</t>
+        </is>
+      </c>
+      <c r="D39" s="34" t="inlineStr">
+        <is>
+          <t>The Girl With The Pilates Mat</t>
+        </is>
+      </c>
+      <c r="E39" s="33" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ouO3_Mwo2lY</t>
+        </is>
+      </c>
+      <c r="F39" s="35" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G39" s="35" t="n">
+        <v>54</v>
+      </c>
+      <c r="H39" s="33" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I39" s="34" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J39" s="34" t="inlineStr">
+        <is>
+          <t>כדור קטן</t>
+        </is>
+      </c>
+      <c r="K39" s="34" t="inlineStr">
+        <is>
+          <t>בינוני</t>
+        </is>
+      </c>
+      <c r="L39" s="34" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M39" s="34" t="inlineStr">
+        <is>
+          <t>בטן וליבה</t>
+        </is>
+      </c>
+      <c r="N39" s="35" t="n">
+        <v>4</v>
+      </c>
+      <c r="O39" s="35" t="n">
+        <v>4</v>
+      </c>
+      <c r="P39" s="35" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q39" s="35" t="n">
+        <v>5</v>
+      </c>
+      <c r="R39" s="35" t="n">
+        <v>4</v>
+      </c>
+      <c r="S39" s="35" t="n">
+        <v>5</v>
+      </c>
+      <c r="T39" s="33" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="U39" s="33" t="inlineStr">
+        <is>
+          <t>לכלול בקטלוג</t>
+        </is>
+      </c>
+      <c r="V39" s="36" t="inlineStr">
+        <is>
+          <t>ערוץ מאושר (Master-level Certified Pilates Instructor). לא תואם משבצת קיימת (משבצת כדור קטן מוגדרת רק למתחילים) - תוכן בונוס. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל (oembed+lengthSeconds); לא נצפה תוכן במלואו.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="13.5" customHeight="1" s="25">
+      <c r="A40" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>30 Minute Full Body Standing Pilates with a Resistance Band | Great Arm &amp; Shoulder Workout!</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>The Girl With The Pilates Mat</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>The Girl With The Pilates Mat</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=o1q8QMXtl2g</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G40" t="n">
+        <v>56</v>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>גומיית רצועה ארוכה</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>כתפיים וזרועות</t>
+        </is>
+      </c>
+      <c r="N40" t="n">
+        <v>4</v>
+      </c>
+      <c r="O40" t="n">
+        <v>4</v>
+      </c>
+      <c r="P40" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q40" t="n">
+        <v>5</v>
+      </c>
+      <c r="R40" t="n">
+        <v>4</v>
+      </c>
+      <c r="S40" t="n">
+        <v>5</v>
+      </c>
+      <c r="T40" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>לכלול בקטלוג</t>
+        </is>
+      </c>
+      <c r="V40" t="inlineStr">
+        <is>
+          <t>ערוץ מאושר (Master-level Certified Pilates Instructor). [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל (oembed+lengthSeconds); לא נצפה תוכן במלואו.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="13.5" customHeight="1" s="25">
+      <c r="A41" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Standing Pilates Full Body Workout with Resistance Band | At Home Pilates | 20 Mins</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>The Girl With The Pilates Mat</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>The Girl With The Pilates Mat</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=FFybrUAvhy0</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G41" t="n">
+        <v>22</v>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>גומיית רצועה ארוכה</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>גוף מלא</t>
+        </is>
+      </c>
+      <c r="N41" t="n">
+        <v>4</v>
+      </c>
+      <c r="O41" t="n">
+        <v>4</v>
+      </c>
+      <c r="P41" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q41" t="n">
+        <v>5</v>
+      </c>
+      <c r="R41" t="n">
+        <v>4</v>
+      </c>
+      <c r="S41" t="n">
+        <v>5</v>
+      </c>
+      <c r="T41" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="U41" t="inlineStr">
+        <is>
+          <t>לכלול בקטלוג</t>
+        </is>
+      </c>
+      <c r="V41" t="inlineStr">
+        <is>
+          <t>ערוץ מאושר (Master-level Certified Pilates Instructor). [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל (oembed+lengthSeconds); לא נצפה תוכן במלואו.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>40 Minute Full Body Pilates Workout with Resistance Band</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>The Girl With The Pilates Mat</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>The Girl With The Pilates Mat</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=OC5vUAMQELQ</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G42" t="n">
+        <v>71</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>גומיית רצועה ארוכה</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>גוף מלא</t>
+        </is>
+      </c>
+      <c r="N42" t="n">
+        <v>4</v>
+      </c>
+      <c r="O42" t="n">
+        <v>4</v>
+      </c>
+      <c r="P42" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q42" t="n">
+        <v>5</v>
+      </c>
+      <c r="R42" t="n">
+        <v>4</v>
+      </c>
+      <c r="S42" t="n">
+        <v>5</v>
+      </c>
+      <c r="T42" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="U42" t="inlineStr">
+        <is>
+          <t>לכלול בקטלוג</t>
+        </is>
+      </c>
+      <c r="V42" t="inlineStr">
+        <is>
+          <t>ערוץ מאושר (Master-level Certified Pilates Instructor). [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל (oembed+lengthSeconds); לא נצפה תוכן במלואו.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>10 Minute Pilates Ring Workout for Inner Thighs &amp; Core | Quick, Effective &amp; Low-Impact</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>The Girl With The Pilates Mat</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>The Girl With The Pilates Mat</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=3xNZTmlwkzk</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G43" t="n">
+        <v>12</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>טבעת פילאטיס (Ring)</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>ישבן ורגליים / בטן וליבה</t>
+        </is>
+      </c>
+      <c r="N43" t="n">
+        <v>4</v>
+      </c>
+      <c r="O43" t="n">
+        <v>4</v>
+      </c>
+      <c r="P43" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q43" t="n">
+        <v>5</v>
+      </c>
+      <c r="R43" t="n">
+        <v>4</v>
+      </c>
+      <c r="S43" t="n">
+        <v>5</v>
+      </c>
+      <c r="T43" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="U43" t="inlineStr">
+        <is>
+          <t>לכלול בקטלוג</t>
+        </is>
+      </c>
+      <c r="V43" t="inlineStr">
+        <is>
+          <t>ערוץ מאושר (Master-level Certified Pilates Instructor). [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל (oembed+lengthSeconds); לא נצפה תוכן במלואו.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Standing Pilates Full Body Workout with Resistance Band for Beginners | 20 Mins</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>The Girl With The Pilates Mat</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>The Girl With The Pilates Mat</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=CoouH7YSrgE</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G44" t="n">
+        <v>19</v>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>גומיית רצועה ארוכה</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>גוף מלא</t>
+        </is>
+      </c>
+      <c r="N44" t="n">
+        <v>4</v>
+      </c>
+      <c r="O44" t="n">
+        <v>4</v>
+      </c>
+      <c r="P44" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q44" t="n">
+        <v>5</v>
+      </c>
+      <c r="R44" t="n">
+        <v>4</v>
+      </c>
+      <c r="S44" t="n">
+        <v>5</v>
+      </c>
+      <c r="T44" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="U44" t="inlineStr">
+        <is>
+          <t>לכלול בקטלוג</t>
+        </is>
+      </c>
+      <c r="V44" t="inlineStr">
+        <is>
+          <t>ערוץ מאושר (Master-level Certified Pilates Instructor). [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל (oembed+lengthSeconds); לא נצפה תוכן במלואו.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Standing Pilates Ring Workout to Tone Arms, Back and Shoulders After 40</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>The Girl With The Pilates Mat</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>The Girl With The Pilates Mat</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ZxLJ8jbnURc</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G45" t="n">
+        <v>15</v>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>טבעת פילאטיס (Ring)</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>כתפיים וזרועות / גב ויציבה</t>
+        </is>
+      </c>
+      <c r="N45" t="n">
+        <v>4</v>
+      </c>
+      <c r="O45" t="n">
+        <v>4</v>
+      </c>
+      <c r="P45" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q45" t="n">
+        <v>5</v>
+      </c>
+      <c r="R45" t="n">
+        <v>4</v>
+      </c>
+      <c r="S45" t="n">
+        <v>5</v>
+      </c>
+      <c r="T45" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="U45" t="inlineStr">
+        <is>
+          <t>לכלול בקטלוג</t>
+        </is>
+      </c>
+      <c r="V45" t="inlineStr">
+        <is>
+          <t>ערוץ מאושר (Master-level Certified Pilates Instructor). [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל (oembed+lengthSeconds); לא נצפה תוכן במלואו.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>15 Min Upper Body Resistance Band Workout for Strong Back, Arms and Shoulders | Pilates Arm Workout</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>The Girl With The Pilates Mat</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>The Girl With The Pilates Mat</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=JdO0B4MkhTM</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G46" t="n">
+        <v>16</v>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>גומיית רצועה ארוכה</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>כתפיים וזרועות / גב ויציבה</t>
+        </is>
+      </c>
+      <c r="N46" t="n">
+        <v>4</v>
+      </c>
+      <c r="O46" t="n">
+        <v>4</v>
+      </c>
+      <c r="P46" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q46" t="n">
+        <v>5</v>
+      </c>
+      <c r="R46" t="n">
+        <v>4</v>
+      </c>
+      <c r="S46" t="n">
+        <v>5</v>
+      </c>
+      <c r="T46" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="U46" t="inlineStr">
+        <is>
+          <t>לכלול בקטלוג</t>
+        </is>
+      </c>
+      <c r="V46" t="inlineStr">
+        <is>
+          <t>ערוץ מאושר (Master-level Certified Pilates Instructor). [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל (oembed+lengthSeconds); לא נצפה תוכן במלואו.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Resistance Band Pilates Workout 25 Min</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>The Girl With The Pilates Mat</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>The Girl With The Pilates Mat</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=bpkB4E4aNNw</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G47" t="n">
+        <v>53</v>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>גומיית רצועה ארוכה</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>גוף מלא</t>
+        </is>
+      </c>
+      <c r="N47" t="n">
+        <v>4</v>
+      </c>
+      <c r="O47" t="n">
+        <v>4</v>
+      </c>
+      <c r="P47" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q47" t="n">
+        <v>5</v>
+      </c>
+      <c r="R47" t="n">
+        <v>4</v>
+      </c>
+      <c r="S47" t="n">
+        <v>5</v>
+      </c>
+      <c r="T47" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="U47" t="inlineStr">
+        <is>
+          <t>לכלול בקטלוג</t>
+        </is>
+      </c>
+      <c r="V47" t="inlineStr">
+        <is>
+          <t>ערוץ מאושר (Master-level Certified Pilates Instructor). [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל (oembed+lengthSeconds); לא נצפה תוכן במלואו.]</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="T2:T41">
     <cfRule type="cellIs" rank="0" priority="2" equalAverage="0" operator="greaterThanOrEqual" aboveAverage="0" dxfId="2" text="" percent="0" bottom="0">
@@ -6917,7 +7934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O42"/>
+  <dimension ref="A1:O47"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6171875" defaultRowHeight="13.5" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="6" customWidth="1" style="24" min="1" max="1"/>
@@ -9457,115 +10474,866 @@
       </c>
     </row>
     <row r="36" ht="13.5" customHeight="1" s="25">
-      <c r="A36" s="33" t="n"/>
-      <c r="B36" s="36" t="n"/>
-      <c r="C36" s="36" t="n"/>
-      <c r="D36" s="34" t="n"/>
-      <c r="E36" s="33" t="n"/>
-      <c r="F36" s="35" t="n"/>
-      <c r="G36" s="33" t="n"/>
-      <c r="H36" s="33" t="n"/>
-      <c r="I36" s="34" t="n"/>
-      <c r="J36" s="34" t="n"/>
-      <c r="K36" s="34" t="n"/>
-      <c r="L36" s="34" t="n"/>
-      <c r="M36" s="34" t="n"/>
-      <c r="N36" s="33" t="n"/>
-      <c r="O36" s="36" t="n"/>
+      <c r="A36" s="33" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="36" t="inlineStr">
+        <is>
+          <t>Pilates Strength Training with a Mini Band | 15 mins Upper Body | 15 Mins Legs, Core &amp; Glutes</t>
+        </is>
+      </c>
+      <c r="C36" s="36" t="inlineStr">
+        <is>
+          <t>The Girl With The Pilates Mat</t>
+        </is>
+      </c>
+      <c r="D36" s="34" t="inlineStr">
+        <is>
+          <t>The Girl With The Pilates Mat</t>
+        </is>
+      </c>
+      <c r="E36" s="33" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=tD8TW3KmBg4</t>
+        </is>
+      </c>
+      <c r="F36" s="35" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G36" s="33" t="n">
+        <v>56</v>
+      </c>
+      <c r="H36" s="33" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I36" s="34" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J36" s="34" t="inlineStr">
+        <is>
+          <t>גומיית לולאה</t>
+        </is>
+      </c>
+      <c r="K36" s="34" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L36" s="34" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M36" s="34" t="inlineStr">
+        <is>
+          <t>כתפיים וזרועות / ישבן ורגליים / בטן וליבה</t>
+        </is>
+      </c>
+      <c r="N36" s="33">
+        <f>'מאגר מועמדים'!T36</f>
+        <v/>
+      </c>
+      <c r="O36" s="36" t="inlineStr">
+        <is>
+          <t>אושר לקטלוג. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל (oembed+lengthSeconds); לא נצפה תוכן במלואו.]</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="13.5" customHeight="1" s="25">
-      <c r="A37" s="33" t="n"/>
-      <c r="B37" s="36" t="n"/>
-      <c r="C37" s="36" t="n"/>
-      <c r="D37" s="34" t="n"/>
-      <c r="E37" s="33" t="n"/>
-      <c r="F37" s="35" t="n"/>
-      <c r="G37" s="33" t="n"/>
-      <c r="H37" s="33" t="n"/>
-      <c r="I37" s="34" t="n"/>
-      <c r="J37" s="34" t="n"/>
-      <c r="K37" s="34" t="n"/>
-      <c r="L37" s="34" t="n"/>
-      <c r="M37" s="34" t="n"/>
-      <c r="N37" s="33" t="n"/>
-      <c r="O37" s="36" t="n"/>
+      <c r="A37" s="33" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="36" t="inlineStr">
+        <is>
+          <t>Pilates Mini Resistance Band Class | 30 Minutes | Full Body Workout</t>
+        </is>
+      </c>
+      <c r="C37" s="36" t="inlineStr">
+        <is>
+          <t>The Girl With The Pilates Mat</t>
+        </is>
+      </c>
+      <c r="D37" s="34" t="inlineStr">
+        <is>
+          <t>The Girl With The Pilates Mat</t>
+        </is>
+      </c>
+      <c r="E37" s="33" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=sh5_uhqLGZw</t>
+        </is>
+      </c>
+      <c r="F37" s="35" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G37" s="33" t="n">
+        <v>48</v>
+      </c>
+      <c r="H37" s="33" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I37" s="34" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J37" s="34" t="inlineStr">
+        <is>
+          <t>גומיית לולאה</t>
+        </is>
+      </c>
+      <c r="K37" s="34" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L37" s="34" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M37" s="34" t="inlineStr">
+        <is>
+          <t>גוף מלא</t>
+        </is>
+      </c>
+      <c r="N37" s="33">
+        <f>'מאגר מועמדים'!T37</f>
+        <v/>
+      </c>
+      <c r="O37" s="36" t="inlineStr">
+        <is>
+          <t>אושר לקטלוג. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל (oembed+lengthSeconds); לא נצפה תוכן במלואו.]</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="13.5" customHeight="1" s="25">
-      <c r="A38" s="33" t="n"/>
-      <c r="B38" s="36" t="n"/>
-      <c r="C38" s="36" t="n"/>
-      <c r="D38" s="34" t="n"/>
-      <c r="E38" s="33" t="n"/>
-      <c r="F38" s="35" t="n"/>
-      <c r="G38" s="33" t="n"/>
-      <c r="H38" s="33" t="n"/>
-      <c r="I38" s="34" t="n"/>
-      <c r="J38" s="34" t="n"/>
-      <c r="K38" s="34" t="n"/>
-      <c r="L38" s="34" t="n"/>
-      <c r="M38" s="34" t="n"/>
-      <c r="N38" s="33" t="n"/>
-      <c r="O38" s="36" t="n"/>
+      <c r="A38" s="33" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="36" t="inlineStr">
+        <is>
+          <t>40 MIN FULL BODY MINI BAND WORKOUT | Intermediate Pilates with Mini Band ( Optional)</t>
+        </is>
+      </c>
+      <c r="C38" s="36" t="inlineStr">
+        <is>
+          <t>The Girl With The Pilates Mat</t>
+        </is>
+      </c>
+      <c r="D38" s="34" t="inlineStr">
+        <is>
+          <t>The Girl With The Pilates Mat</t>
+        </is>
+      </c>
+      <c r="E38" s="33" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=F2iru_IAqJ0</t>
+        </is>
+      </c>
+      <c r="F38" s="35" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G38" s="33" t="n">
+        <v>72</v>
+      </c>
+      <c r="H38" s="33" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I38" s="34" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J38" s="34" t="inlineStr">
+        <is>
+          <t>גומיית לולאה</t>
+        </is>
+      </c>
+      <c r="K38" s="34" t="inlineStr">
+        <is>
+          <t>בינוני</t>
+        </is>
+      </c>
+      <c r="L38" s="34" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M38" s="34" t="inlineStr">
+        <is>
+          <t>גוף מלא</t>
+        </is>
+      </c>
+      <c r="N38" s="33">
+        <f>'מאגר מועמדים'!T38</f>
+        <v/>
+      </c>
+      <c r="O38" s="36" t="inlineStr">
+        <is>
+          <t>אושר לקטלוג. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל (oembed+lengthSeconds); לא נצפה תוכן במלואו.]</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="13.5" customHeight="1" s="25">
-      <c r="A39" s="33" t="n"/>
-      <c r="B39" s="36" t="n"/>
-      <c r="C39" s="36" t="n"/>
-      <c r="D39" s="34" t="n"/>
-      <c r="E39" s="33" t="n"/>
-      <c r="F39" s="35" t="n"/>
-      <c r="G39" s="33" t="n"/>
-      <c r="H39" s="33" t="n"/>
-      <c r="I39" s="34" t="n"/>
-      <c r="J39" s="34" t="n"/>
-      <c r="K39" s="34" t="n"/>
-      <c r="L39" s="34" t="n"/>
-      <c r="M39" s="34" t="n"/>
-      <c r="N39" s="33" t="n"/>
-      <c r="O39" s="36" t="n"/>
+      <c r="A39" s="33" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="36" t="inlineStr">
+        <is>
+          <t>Pilates Mini Ball Workout for Core Strength and Stability | Intermediate Level | 30 Min</t>
+        </is>
+      </c>
+      <c r="C39" s="36" t="inlineStr">
+        <is>
+          <t>The Girl With The Pilates Mat</t>
+        </is>
+      </c>
+      <c r="D39" s="34" t="inlineStr">
+        <is>
+          <t>The Girl With The Pilates Mat</t>
+        </is>
+      </c>
+      <c r="E39" s="33" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ouO3_Mwo2lY</t>
+        </is>
+      </c>
+      <c r="F39" s="35" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G39" s="33" t="n">
+        <v>54</v>
+      </c>
+      <c r="H39" s="33" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I39" s="34" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J39" s="34" t="inlineStr">
+        <is>
+          <t>כדור קטן</t>
+        </is>
+      </c>
+      <c r="K39" s="34" t="inlineStr">
+        <is>
+          <t>בינוני</t>
+        </is>
+      </c>
+      <c r="L39" s="34" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M39" s="34" t="inlineStr">
+        <is>
+          <t>בטן וליבה</t>
+        </is>
+      </c>
+      <c r="N39" s="33">
+        <f>'מאגר מועמדים'!T39</f>
+        <v/>
+      </c>
+      <c r="O39" s="36" t="inlineStr">
+        <is>
+          <t>אושר לקטלוג. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל (oembed+lengthSeconds); לא נצפה תוכן במלואו.]</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="13.5" customHeight="1" s="25">
-      <c r="A40" s="33" t="n"/>
-      <c r="B40" s="36" t="n"/>
-      <c r="C40" s="36" t="n"/>
-      <c r="D40" s="34" t="n"/>
-      <c r="E40" s="33" t="n"/>
-      <c r="F40" s="35" t="n"/>
-      <c r="G40" s="33" t="n"/>
-      <c r="H40" s="33" t="n"/>
-      <c r="I40" s="34" t="n"/>
-      <c r="J40" s="34" t="n"/>
-      <c r="K40" s="34" t="n"/>
-      <c r="L40" s="34" t="n"/>
-      <c r="M40" s="34" t="n"/>
-      <c r="N40" s="33" t="n"/>
-      <c r="O40" s="36" t="n"/>
+      <c r="A40" s="33" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="36" t="inlineStr">
+        <is>
+          <t>30 Minute Full Body Standing Pilates with a Resistance Band | Great Arm &amp; Shoulder Workout!</t>
+        </is>
+      </c>
+      <c r="C40" s="36" t="inlineStr">
+        <is>
+          <t>The Girl With The Pilates Mat</t>
+        </is>
+      </c>
+      <c r="D40" s="34" t="inlineStr">
+        <is>
+          <t>The Girl With The Pilates Mat</t>
+        </is>
+      </c>
+      <c r="E40" s="33" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=o1q8QMXtl2g</t>
+        </is>
+      </c>
+      <c r="F40" s="35" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G40" s="33" t="n">
+        <v>56</v>
+      </c>
+      <c r="H40" s="33" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I40" s="34" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J40" s="34" t="inlineStr">
+        <is>
+          <t>גומיית רצועה ארוכה</t>
+        </is>
+      </c>
+      <c r="K40" s="34" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L40" s="34" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M40" s="34" t="inlineStr">
+        <is>
+          <t>כתפיים וזרועות</t>
+        </is>
+      </c>
+      <c r="N40" s="33">
+        <f>'מאגר מועמדים'!T40</f>
+        <v/>
+      </c>
+      <c r="O40" s="36" t="inlineStr">
+        <is>
+          <t>אושר לקטלוג. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל (oembed+lengthSeconds); לא נצפה תוכן במלואו.]</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="13.5" customHeight="1" s="25">
-      <c r="A41" s="33" t="n"/>
-      <c r="B41" s="36" t="n"/>
-      <c r="C41" s="36" t="n"/>
-      <c r="D41" s="34" t="n"/>
-      <c r="E41" s="33" t="n"/>
-      <c r="F41" s="35" t="n"/>
-      <c r="G41" s="33" t="n"/>
-      <c r="H41" s="33" t="n"/>
-      <c r="I41" s="34" t="n"/>
-      <c r="J41" s="34" t="n"/>
-      <c r="K41" s="34" t="n"/>
-      <c r="L41" s="34" t="n"/>
-      <c r="M41" s="34" t="n"/>
-      <c r="N41" s="33" t="n"/>
-      <c r="O41" s="36" t="n"/>
+      <c r="A41" s="33" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="36" t="inlineStr">
+        <is>
+          <t>Standing Pilates Full Body Workout with Resistance Band | At Home Pilates | 20 Mins</t>
+        </is>
+      </c>
+      <c r="C41" s="36" t="inlineStr">
+        <is>
+          <t>The Girl With The Pilates Mat</t>
+        </is>
+      </c>
+      <c r="D41" s="34" t="inlineStr">
+        <is>
+          <t>The Girl With The Pilates Mat</t>
+        </is>
+      </c>
+      <c r="E41" s="33" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=FFybrUAvhy0</t>
+        </is>
+      </c>
+      <c r="F41" s="35" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G41" s="33" t="n">
+        <v>22</v>
+      </c>
+      <c r="H41" s="33" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I41" s="34" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J41" s="34" t="inlineStr">
+        <is>
+          <t>גומיית רצועה ארוכה</t>
+        </is>
+      </c>
+      <c r="K41" s="34" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L41" s="34" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M41" s="34" t="inlineStr">
+        <is>
+          <t>גוף מלא</t>
+        </is>
+      </c>
+      <c r="N41" s="33">
+        <f>'מאגר מועמדים'!T41</f>
+        <v/>
+      </c>
+      <c r="O41" s="36" t="inlineStr">
+        <is>
+          <t>אושר לקטלוג. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל (oembed+lengthSeconds); לא נצפה תוכן במלואו.]</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="13.5" customHeight="1" s="25">
-      <c r="A42" s="37">
-        <f>COUNTA(B2:B41)</f>
+      <c r="A42" s="37" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="37" t="inlineStr">
+        <is>
+          <t>40 Minute Full Body Pilates Workout with Resistance Band</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>The Girl With The Pilates Mat</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>The Girl With The Pilates Mat</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=OC5vUAMQELQ</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G42" t="n">
+        <v>71</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>גומיית רצועה ארוכה</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>גוף מלא</t>
+        </is>
+      </c>
+      <c r="N42">
+        <f>'מאגר מועמדים'!T42</f>
         <v/>
       </c>
-      <c r="B42" s="37" t="inlineStr">
-        <is>
-          <t>סה"כ פריטים בקטלוג</t>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>אושר לקטלוג. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל (oembed+lengthSeconds); לא נצפה תוכן במלואו.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>10 Minute Pilates Ring Workout for Inner Thighs &amp; Core | Quick, Effective &amp; Low-Impact</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>The Girl With The Pilates Mat</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>The Girl With The Pilates Mat</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=3xNZTmlwkzk</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G43" t="n">
+        <v>12</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>טבעת פילאטיס (Ring)</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>ישבן ורגליים / בטן וליבה</t>
+        </is>
+      </c>
+      <c r="N43">
+        <f>'מאגר מועמדים'!T43</f>
+        <v/>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>אושר לקטלוג. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל (oembed+lengthSeconds); לא נצפה תוכן במלואו.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Standing Pilates Full Body Workout with Resistance Band for Beginners | 20 Mins</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>The Girl With The Pilates Mat</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>The Girl With The Pilates Mat</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=CoouH7YSrgE</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G44" t="n">
+        <v>19</v>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>גומיית רצועה ארוכה</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>גוף מלא</t>
+        </is>
+      </c>
+      <c r="N44">
+        <f>'מאגר מועמדים'!T44</f>
+        <v/>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>אושר לקטלוג. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל (oembed+lengthSeconds); לא נצפה תוכן במלואו.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Standing Pilates Ring Workout to Tone Arms, Back and Shoulders After 40</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>The Girl With The Pilates Mat</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>The Girl With The Pilates Mat</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=ZxLJ8jbnURc</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G45" t="n">
+        <v>15</v>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>טבעת פילאטיס (Ring)</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>כתפיים וזרועות / גב ויציבה</t>
+        </is>
+      </c>
+      <c r="N45">
+        <f>'מאגר מועמדים'!T45</f>
+        <v/>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>אושר לקטלוג. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל (oembed+lengthSeconds); לא נצפה תוכן במלואו.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>15 Min Upper Body Resistance Band Workout for Strong Back, Arms and Shoulders | Pilates Arm Workout</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>The Girl With The Pilates Mat</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>The Girl With The Pilates Mat</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=JdO0B4MkhTM</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G46" t="n">
+        <v>16</v>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>גומיית רצועה ארוכה</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>כתפיים וזרועות / גב ויציבה</t>
+        </is>
+      </c>
+      <c r="N46">
+        <f>'מאגר מועמדים'!T46</f>
+        <v/>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>אושר לקטלוג. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל (oembed+lengthSeconds); לא נצפה תוכן במלואו.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Resistance Band Pilates Workout 25 Min</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>The Girl With The Pilates Mat</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>The Girl With The Pilates Mat</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=bpkB4E4aNNw</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G47" t="n">
+        <v>53</v>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>גומיית רצועה ארוכה</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>גוף מלא</t>
+        </is>
+      </c>
+      <c r="N47">
+        <f>'מאגר מועמדים'!T47</f>
+        <v/>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>אושר לקטלוג. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל (oembed+lengthSeconds); לא נצפה תוכן במלואו.]</t>
         </is>
       </c>
     </row>
@@ -10753,37 +12521,37 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="n">
+      <c r="A21" s="24" t="n">
         <v>20</v>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="24" t="inlineStr">
         <is>
           <t>British Heart Foundation</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C21" s="24" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@britishheartfoundation</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D21" s="24" t="inlineStr">
         <is>
           <t>מאושר</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr">
+      <c r="E21" s="24" t="inlineStr">
         <is>
           <t>תוכן פעילות גופנית/גומיות התנגדות לבריאות הלב (לא ערוץ פילאטיס ייעודי)</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="F21" s="24" t="inlineStr">
         <is>
           <t>עמותת בריאות לאומית מובילה בבריטניה (לא הסמכת פילאטיס אישית)</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
-      <c r="I21" t="inlineStr">
+      <c r="G21" s="24" t="inlineStr"/>
+      <c r="H21" s="24" t="inlineStr"/>
+      <c r="I21" s="24" t="inlineStr">
         <is>
           <t>נוסף ע"י Claude, 30.08.2026 - אותר דרך סרטון ספציפי שביקש המשתמש. 114K מנויים, 1,118 סרטונים - עמותה רפואית מוכרת ומבוססת (לא מדריך/ה עצמאי/ת), רמת אמינות גבוהה מאוד למרות שאינה "ערוץ פילאטיס" במובן הרגיל - תוכן פעילות גופנית/שיקום לב מבוסס-בטיחות.</t>
         </is>

</xml_diff>

<commit_message>
Fix broken Jessica Valant channel URL in approved-channels sheet
</commit_message>
<xml_diff>
--- a/YR1/pilates/data/מטריצת_כיסוי_קטלוג_פילאטיס_v5.xlsx
+++ b/YR1/pilates/data/מטריצת_כיסוי_קטלוג_פילאטיס_v5.xlsx
@@ -955,7 +955,7 @@
       </c>
     </row>
     <row r="54">
-      <c r="A54" t="inlineStr">
+      <c r="A54" s="24" t="inlineStr">
         <is>
           <t>• 30.08.2026: עברתי על סרטוני הערוץ "The Girl With The Pilates Mat" לבקשת המשתמש - נוספו 12 סרטונים חדשים (#35-46). סגרו לגמרי: #7,#13,#25,#26 (הושלמו); הרחיבו משמעותית: #4,#24,#28 (חלקי); #29 עבר את היעד בהרבה (מותר לפי הנחיית המשתמש). 2 סרטונים (בינוני/כדור-קטן-בינוני) לא תאמו משבצת קיימת - נוספו כתוכן בונוס.</t>
         </is>
@@ -7113,752 +7113,752 @@
       </c>
     </row>
     <row r="40" ht="13.5" customHeight="1" s="25">
-      <c r="A40" t="n">
+      <c r="A40" s="24" t="n">
         <v>39</v>
       </c>
-      <c r="B40" t="inlineStr">
+      <c r="B40" s="24" t="inlineStr">
         <is>
           <t>30 Minute Full Body Standing Pilates with a Resistance Band | Great Arm &amp; Shoulder Workout!</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr">
+      <c r="C40" s="24" t="inlineStr">
         <is>
           <t>The Girl With The Pilates Mat</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr">
+      <c r="D40" s="24" t="inlineStr">
         <is>
           <t>The Girl With The Pilates Mat</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr">
+      <c r="E40" s="24" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=o1q8QMXtl2g</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr">
+      <c r="F40" s="24" t="inlineStr">
         <is>
           <t>לא אומת</t>
         </is>
       </c>
-      <c r="G40" t="n">
+      <c r="G40" s="24" t="n">
         <v>56</v>
       </c>
-      <c r="H40" t="inlineStr">
+      <c r="H40" s="24" t="inlineStr">
         <is>
           <t>אנגלית</t>
         </is>
       </c>
-      <c r="I40" t="inlineStr">
+      <c r="I40" s="24" t="inlineStr">
         <is>
           <t>תרגיל</t>
         </is>
       </c>
-      <c r="J40" t="inlineStr">
+      <c r="J40" s="24" t="inlineStr">
         <is>
           <t>גומיית רצועה ארוכה</t>
         </is>
       </c>
-      <c r="K40" t="inlineStr">
+      <c r="K40" s="24" t="inlineStr">
         <is>
           <t>מתחילים</t>
         </is>
       </c>
-      <c r="L40" t="inlineStr">
+      <c r="L40" s="24" t="inlineStr">
         <is>
           <t>חיזוק</t>
         </is>
       </c>
-      <c r="M40" t="inlineStr">
+      <c r="M40" s="24" t="inlineStr">
         <is>
           <t>כתפיים וזרועות</t>
         </is>
       </c>
-      <c r="N40" t="n">
-        <v>4</v>
-      </c>
-      <c r="O40" t="n">
-        <v>4</v>
-      </c>
-      <c r="P40" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q40" t="n">
+      <c r="N40" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="O40" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="P40" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q40" s="24" t="n">
         <v>5</v>
       </c>
-      <c r="R40" t="n">
-        <v>4</v>
-      </c>
-      <c r="S40" t="n">
+      <c r="R40" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="S40" s="24" t="n">
         <v>5</v>
       </c>
-      <c r="T40" t="n">
+      <c r="T40" s="24" t="n">
         <v>4.3</v>
       </c>
-      <c r="U40" t="inlineStr">
+      <c r="U40" s="24" t="inlineStr">
         <is>
           <t>לכלול בקטלוג</t>
         </is>
       </c>
-      <c r="V40" t="inlineStr">
+      <c r="V40" s="24" t="inlineStr">
         <is>
           <t>ערוץ מאושר (Master-level Certified Pilates Instructor). [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל (oembed+lengthSeconds); לא נצפה תוכן במלואו.]</t>
         </is>
       </c>
     </row>
     <row r="41" ht="13.5" customHeight="1" s="25">
-      <c r="A41" t="n">
+      <c r="A41" s="24" t="n">
         <v>40</v>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B41" s="24" t="inlineStr">
         <is>
           <t>Standing Pilates Full Body Workout with Resistance Band | At Home Pilates | 20 Mins</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C41" s="24" t="inlineStr">
         <is>
           <t>The Girl With The Pilates Mat</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D41" s="24" t="inlineStr">
         <is>
           <t>The Girl With The Pilates Mat</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
+      <c r="E41" s="24" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=FFybrUAvhy0</t>
         </is>
       </c>
-      <c r="F41" t="inlineStr">
+      <c r="F41" s="24" t="inlineStr">
         <is>
           <t>לא אומת</t>
         </is>
       </c>
-      <c r="G41" t="n">
+      <c r="G41" s="24" t="n">
         <v>22</v>
       </c>
-      <c r="H41" t="inlineStr">
+      <c r="H41" s="24" t="inlineStr">
         <is>
           <t>אנגלית</t>
         </is>
       </c>
-      <c r="I41" t="inlineStr">
+      <c r="I41" s="24" t="inlineStr">
         <is>
           <t>תרגיל</t>
         </is>
       </c>
-      <c r="J41" t="inlineStr">
+      <c r="J41" s="24" t="inlineStr">
         <is>
           <t>גומיית רצועה ארוכה</t>
         </is>
       </c>
-      <c r="K41" t="inlineStr">
+      <c r="K41" s="24" t="inlineStr">
         <is>
           <t>מתחילים</t>
         </is>
       </c>
-      <c r="L41" t="inlineStr">
+      <c r="L41" s="24" t="inlineStr">
         <is>
           <t>חיזוק</t>
         </is>
       </c>
-      <c r="M41" t="inlineStr">
+      <c r="M41" s="24" t="inlineStr">
         <is>
           <t>גוף מלא</t>
         </is>
       </c>
-      <c r="N41" t="n">
-        <v>4</v>
-      </c>
-      <c r="O41" t="n">
-        <v>4</v>
-      </c>
-      <c r="P41" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q41" t="n">
+      <c r="N41" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="O41" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="P41" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q41" s="24" t="n">
         <v>5</v>
       </c>
-      <c r="R41" t="n">
-        <v>4</v>
-      </c>
-      <c r="S41" t="n">
+      <c r="R41" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="S41" s="24" t="n">
         <v>5</v>
       </c>
-      <c r="T41" t="n">
+      <c r="T41" s="24" t="n">
         <v>4.3</v>
       </c>
-      <c r="U41" t="inlineStr">
+      <c r="U41" s="24" t="inlineStr">
         <is>
           <t>לכלול בקטלוג</t>
         </is>
       </c>
-      <c r="V41" t="inlineStr">
+      <c r="V41" s="24" t="inlineStr">
         <is>
           <t>ערוץ מאושר (Master-level Certified Pilates Instructor). [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל (oembed+lengthSeconds); לא נצפה תוכן במלואו.]</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" t="n">
+      <c r="A42" s="24" t="n">
         <v>41</v>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="B42" s="24" t="inlineStr">
         <is>
           <t>40 Minute Full Body Pilates Workout with Resistance Band</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C42" s="24" t="inlineStr">
         <is>
           <t>The Girl With The Pilates Mat</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="D42" s="24" t="inlineStr">
         <is>
           <t>The Girl With The Pilates Mat</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="E42" s="24" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=OC5vUAMQELQ</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr">
+      <c r="F42" s="24" t="inlineStr">
         <is>
           <t>לא אומת</t>
         </is>
       </c>
-      <c r="G42" t="n">
+      <c r="G42" s="24" t="n">
         <v>71</v>
       </c>
-      <c r="H42" t="inlineStr">
+      <c r="H42" s="24" t="inlineStr">
         <is>
           <t>אנגלית</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr">
+      <c r="I42" s="24" t="inlineStr">
         <is>
           <t>תרגיל</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr">
+      <c r="J42" s="24" t="inlineStr">
         <is>
           <t>גומיית רצועה ארוכה</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr">
+      <c r="K42" s="24" t="inlineStr">
         <is>
           <t>מתחילים</t>
         </is>
       </c>
-      <c r="L42" t="inlineStr">
+      <c r="L42" s="24" t="inlineStr">
         <is>
           <t>חיזוק</t>
         </is>
       </c>
-      <c r="M42" t="inlineStr">
+      <c r="M42" s="24" t="inlineStr">
         <is>
           <t>גוף מלא</t>
         </is>
       </c>
-      <c r="N42" t="n">
-        <v>4</v>
-      </c>
-      <c r="O42" t="n">
-        <v>4</v>
-      </c>
-      <c r="P42" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q42" t="n">
+      <c r="N42" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="O42" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="P42" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q42" s="24" t="n">
         <v>5</v>
       </c>
-      <c r="R42" t="n">
-        <v>4</v>
-      </c>
-      <c r="S42" t="n">
+      <c r="R42" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="S42" s="24" t="n">
         <v>5</v>
       </c>
-      <c r="T42" t="n">
+      <c r="T42" s="24" t="n">
         <v>4.3</v>
       </c>
-      <c r="U42" t="inlineStr">
+      <c r="U42" s="24" t="inlineStr">
         <is>
           <t>לכלול בקטלוג</t>
         </is>
       </c>
-      <c r="V42" t="inlineStr">
+      <c r="V42" s="24" t="inlineStr">
         <is>
           <t>ערוץ מאושר (Master-level Certified Pilates Instructor). [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל (oembed+lengthSeconds); לא נצפה תוכן במלואו.]</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="n">
+      <c r="A43" s="24" t="n">
         <v>42</v>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B43" s="24" t="inlineStr">
         <is>
           <t>10 Minute Pilates Ring Workout for Inner Thighs &amp; Core | Quick, Effective &amp; Low-Impact</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C43" s="24" t="inlineStr">
         <is>
           <t>The Girl With The Pilates Mat</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="D43" s="24" t="inlineStr">
         <is>
           <t>The Girl With The Pilates Mat</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
+      <c r="E43" s="24" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=3xNZTmlwkzk</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr">
+      <c r="F43" s="24" t="inlineStr">
         <is>
           <t>לא אומת</t>
         </is>
       </c>
-      <c r="G43" t="n">
+      <c r="G43" s="24" t="n">
         <v>12</v>
       </c>
-      <c r="H43" t="inlineStr">
+      <c r="H43" s="24" t="inlineStr">
         <is>
           <t>אנגלית</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr">
+      <c r="I43" s="24" t="inlineStr">
         <is>
           <t>תרגיל</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr">
+      <c r="J43" s="24" t="inlineStr">
         <is>
           <t>טבעת פילאטיס (Ring)</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr">
+      <c r="K43" s="24" t="inlineStr">
         <is>
           <t>מתחילים</t>
         </is>
       </c>
-      <c r="L43" t="inlineStr">
+      <c r="L43" s="24" t="inlineStr">
         <is>
           <t>חיזוק</t>
         </is>
       </c>
-      <c r="M43" t="inlineStr">
+      <c r="M43" s="24" t="inlineStr">
         <is>
           <t>ישבן ורגליים / בטן וליבה</t>
         </is>
       </c>
-      <c r="N43" t="n">
-        <v>4</v>
-      </c>
-      <c r="O43" t="n">
-        <v>4</v>
-      </c>
-      <c r="P43" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q43" t="n">
+      <c r="N43" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="O43" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="P43" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q43" s="24" t="n">
         <v>5</v>
       </c>
-      <c r="R43" t="n">
-        <v>4</v>
-      </c>
-      <c r="S43" t="n">
+      <c r="R43" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="S43" s="24" t="n">
         <v>5</v>
       </c>
-      <c r="T43" t="n">
+      <c r="T43" s="24" t="n">
         <v>4.3</v>
       </c>
-      <c r="U43" t="inlineStr">
+      <c r="U43" s="24" t="inlineStr">
         <is>
           <t>לכלול בקטלוג</t>
         </is>
       </c>
-      <c r="V43" t="inlineStr">
+      <c r="V43" s="24" t="inlineStr">
         <is>
           <t>ערוץ מאושר (Master-level Certified Pilates Instructor). [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל (oembed+lengthSeconds); לא נצפה תוכן במלואו.]</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="n">
+      <c r="A44" s="24" t="n">
         <v>43</v>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="B44" s="24" t="inlineStr">
         <is>
           <t>Standing Pilates Full Body Workout with Resistance Band for Beginners | 20 Mins</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C44" s="24" t="inlineStr">
         <is>
           <t>The Girl With The Pilates Mat</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="D44" s="24" t="inlineStr">
         <is>
           <t>The Girl With The Pilates Mat</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr">
+      <c r="E44" s="24" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=CoouH7YSrgE</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr">
+      <c r="F44" s="24" t="inlineStr">
         <is>
           <t>לא אומת</t>
         </is>
       </c>
-      <c r="G44" t="n">
+      <c r="G44" s="24" t="n">
         <v>19</v>
       </c>
-      <c r="H44" t="inlineStr">
+      <c r="H44" s="24" t="inlineStr">
         <is>
           <t>אנגלית</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr">
+      <c r="I44" s="24" t="inlineStr">
         <is>
           <t>תרגיל</t>
         </is>
       </c>
-      <c r="J44" t="inlineStr">
+      <c r="J44" s="24" t="inlineStr">
         <is>
           <t>גומיית רצועה ארוכה</t>
         </is>
       </c>
-      <c r="K44" t="inlineStr">
+      <c r="K44" s="24" t="inlineStr">
         <is>
           <t>מתחילים</t>
         </is>
       </c>
-      <c r="L44" t="inlineStr">
+      <c r="L44" s="24" t="inlineStr">
         <is>
           <t>חיזוק</t>
         </is>
       </c>
-      <c r="M44" t="inlineStr">
+      <c r="M44" s="24" t="inlineStr">
         <is>
           <t>גוף מלא</t>
         </is>
       </c>
-      <c r="N44" t="n">
-        <v>4</v>
-      </c>
-      <c r="O44" t="n">
-        <v>4</v>
-      </c>
-      <c r="P44" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q44" t="n">
+      <c r="N44" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="O44" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="P44" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q44" s="24" t="n">
         <v>5</v>
       </c>
-      <c r="R44" t="n">
-        <v>4</v>
-      </c>
-      <c r="S44" t="n">
+      <c r="R44" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="S44" s="24" t="n">
         <v>5</v>
       </c>
-      <c r="T44" t="n">
+      <c r="T44" s="24" t="n">
         <v>4.3</v>
       </c>
-      <c r="U44" t="inlineStr">
+      <c r="U44" s="24" t="inlineStr">
         <is>
           <t>לכלול בקטלוג</t>
         </is>
       </c>
-      <c r="V44" t="inlineStr">
+      <c r="V44" s="24" t="inlineStr">
         <is>
           <t>ערוץ מאושר (Master-level Certified Pilates Instructor). [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל (oembed+lengthSeconds); לא נצפה תוכן במלואו.]</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="n">
+      <c r="A45" s="24" t="n">
         <v>44</v>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B45" s="24" t="inlineStr">
         <is>
           <t>Standing Pilates Ring Workout to Tone Arms, Back and Shoulders After 40</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C45" s="24" t="inlineStr">
         <is>
           <t>The Girl With The Pilates Mat</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D45" s="24" t="inlineStr">
         <is>
           <t>The Girl With The Pilates Mat</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
+      <c r="E45" s="24" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=ZxLJ8jbnURc</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr">
+      <c r="F45" s="24" t="inlineStr">
         <is>
           <t>לא אומת</t>
         </is>
       </c>
-      <c r="G45" t="n">
+      <c r="G45" s="24" t="n">
         <v>15</v>
       </c>
-      <c r="H45" t="inlineStr">
+      <c r="H45" s="24" t="inlineStr">
         <is>
           <t>אנגלית</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr">
+      <c r="I45" s="24" t="inlineStr">
         <is>
           <t>תרגיל</t>
         </is>
       </c>
-      <c r="J45" t="inlineStr">
+      <c r="J45" s="24" t="inlineStr">
         <is>
           <t>טבעת פילאטיס (Ring)</t>
         </is>
       </c>
-      <c r="K45" t="inlineStr">
+      <c r="K45" s="24" t="inlineStr">
         <is>
           <t>מתחילים</t>
         </is>
       </c>
-      <c r="L45" t="inlineStr">
+      <c r="L45" s="24" t="inlineStr">
         <is>
           <t>חיזוק</t>
         </is>
       </c>
-      <c r="M45" t="inlineStr">
+      <c r="M45" s="24" t="inlineStr">
         <is>
           <t>כתפיים וזרועות / גב ויציבה</t>
         </is>
       </c>
-      <c r="N45" t="n">
-        <v>4</v>
-      </c>
-      <c r="O45" t="n">
-        <v>4</v>
-      </c>
-      <c r="P45" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q45" t="n">
+      <c r="N45" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="O45" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="P45" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q45" s="24" t="n">
         <v>5</v>
       </c>
-      <c r="R45" t="n">
-        <v>4</v>
-      </c>
-      <c r="S45" t="n">
+      <c r="R45" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="S45" s="24" t="n">
         <v>5</v>
       </c>
-      <c r="T45" t="n">
+      <c r="T45" s="24" t="n">
         <v>4.3</v>
       </c>
-      <c r="U45" t="inlineStr">
+      <c r="U45" s="24" t="inlineStr">
         <is>
           <t>לכלול בקטלוג</t>
         </is>
       </c>
-      <c r="V45" t="inlineStr">
+      <c r="V45" s="24" t="inlineStr">
         <is>
           <t>ערוץ מאושר (Master-level Certified Pilates Instructor). [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל (oembed+lengthSeconds); לא נצפה תוכן במלואו.]</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="n">
+      <c r="A46" s="24" t="n">
         <v>45</v>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="B46" s="24" t="inlineStr">
         <is>
           <t>15 Min Upper Body Resistance Band Workout for Strong Back, Arms and Shoulders | Pilates Arm Workout</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C46" s="24" t="inlineStr">
         <is>
           <t>The Girl With The Pilates Mat</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="D46" s="24" t="inlineStr">
         <is>
           <t>The Girl With The Pilates Mat</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr">
+      <c r="E46" s="24" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=JdO0B4MkhTM</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr">
+      <c r="F46" s="24" t="inlineStr">
         <is>
           <t>לא אומת</t>
         </is>
       </c>
-      <c r="G46" t="n">
+      <c r="G46" s="24" t="n">
         <v>16</v>
       </c>
-      <c r="H46" t="inlineStr">
+      <c r="H46" s="24" t="inlineStr">
         <is>
           <t>אנגלית</t>
         </is>
       </c>
-      <c r="I46" t="inlineStr">
+      <c r="I46" s="24" t="inlineStr">
         <is>
           <t>תרגיל</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr">
+      <c r="J46" s="24" t="inlineStr">
         <is>
           <t>גומיית רצועה ארוכה</t>
         </is>
       </c>
-      <c r="K46" t="inlineStr">
+      <c r="K46" s="24" t="inlineStr">
         <is>
           <t>מתחילים</t>
         </is>
       </c>
-      <c r="L46" t="inlineStr">
+      <c r="L46" s="24" t="inlineStr">
         <is>
           <t>חיזוק</t>
         </is>
       </c>
-      <c r="M46" t="inlineStr">
+      <c r="M46" s="24" t="inlineStr">
         <is>
           <t>כתפיים וזרועות / גב ויציבה</t>
         </is>
       </c>
-      <c r="N46" t="n">
-        <v>4</v>
-      </c>
-      <c r="O46" t="n">
-        <v>4</v>
-      </c>
-      <c r="P46" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q46" t="n">
+      <c r="N46" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="O46" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="P46" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q46" s="24" t="n">
         <v>5</v>
       </c>
-      <c r="R46" t="n">
-        <v>4</v>
-      </c>
-      <c r="S46" t="n">
+      <c r="R46" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="S46" s="24" t="n">
         <v>5</v>
       </c>
-      <c r="T46" t="n">
+      <c r="T46" s="24" t="n">
         <v>4.3</v>
       </c>
-      <c r="U46" t="inlineStr">
+      <c r="U46" s="24" t="inlineStr">
         <is>
           <t>לכלול בקטלוג</t>
         </is>
       </c>
-      <c r="V46" t="inlineStr">
+      <c r="V46" s="24" t="inlineStr">
         <is>
           <t>ערוץ מאושר (Master-level Certified Pilates Instructor). [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל (oembed+lengthSeconds); לא נצפה תוכן במלואו.]</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="n">
+      <c r="A47" s="24" t="n">
         <v>46</v>
       </c>
-      <c r="B47" t="inlineStr">
+      <c r="B47" s="24" t="inlineStr">
         <is>
           <t>Resistance Band Pilates Workout 25 Min</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C47" s="24" t="inlineStr">
         <is>
           <t>The Girl With The Pilates Mat</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="D47" s="24" t="inlineStr">
         <is>
           <t>The Girl With The Pilates Mat</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
+      <c r="E47" s="24" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=bpkB4E4aNNw</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr">
+      <c r="F47" s="24" t="inlineStr">
         <is>
           <t>לא אומת</t>
         </is>
       </c>
-      <c r="G47" t="n">
+      <c r="G47" s="24" t="n">
         <v>53</v>
       </c>
-      <c r="H47" t="inlineStr">
+      <c r="H47" s="24" t="inlineStr">
         <is>
           <t>אנגלית</t>
         </is>
       </c>
-      <c r="I47" t="inlineStr">
+      <c r="I47" s="24" t="inlineStr">
         <is>
           <t>תרגיל</t>
         </is>
       </c>
-      <c r="J47" t="inlineStr">
+      <c r="J47" s="24" t="inlineStr">
         <is>
           <t>גומיית רצועה ארוכה</t>
         </is>
       </c>
-      <c r="K47" t="inlineStr">
+      <c r="K47" s="24" t="inlineStr">
         <is>
           <t>מתחילים</t>
         </is>
       </c>
-      <c r="L47" t="inlineStr">
+      <c r="L47" s="24" t="inlineStr">
         <is>
           <t>חיזוק</t>
         </is>
       </c>
-      <c r="M47" t="inlineStr">
+      <c r="M47" s="24" t="inlineStr">
         <is>
           <t>גוף מלא</t>
         </is>
       </c>
-      <c r="N47" t="n">
-        <v>4</v>
-      </c>
-      <c r="O47" t="n">
-        <v>4</v>
-      </c>
-      <c r="P47" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q47" t="n">
+      <c r="N47" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="O47" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="P47" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q47" s="24" t="n">
         <v>5</v>
       </c>
-      <c r="R47" t="n">
-        <v>4</v>
-      </c>
-      <c r="S47" t="n">
+      <c r="R47" s="24" t="n">
+        <v>4</v>
+      </c>
+      <c r="S47" s="24" t="n">
         <v>5</v>
       </c>
-      <c r="T47" t="n">
+      <c r="T47" s="24" t="n">
         <v>4.3</v>
       </c>
-      <c r="U47" t="inlineStr">
+      <c r="U47" s="24" t="inlineStr">
         <is>
           <t>לכלול בקטלוג</t>
         </is>
       </c>
-      <c r="V47" t="inlineStr">
+      <c r="V47" s="24" t="inlineStr">
         <is>
           <t>ערוץ מאושר (Master-level Certified Pilates Instructor). [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל (oembed+lengthSeconds); לא נצפה תוכן במלואו.]</t>
         </is>
@@ -10914,424 +10914,424 @@
           <t>40 Minute Full Body Pilates Workout with Resistance Band</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
+      <c r="C42" s="24" t="inlineStr">
         <is>
           <t>The Girl With The Pilates Mat</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
+      <c r="D42" s="24" t="inlineStr">
         <is>
           <t>The Girl With The Pilates Mat</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr">
+      <c r="E42" s="24" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=OC5vUAMQELQ</t>
         </is>
       </c>
-      <c r="F42" t="inlineStr">
+      <c r="F42" s="24" t="inlineStr">
         <is>
           <t>לא אומת</t>
         </is>
       </c>
-      <c r="G42" t="n">
+      <c r="G42" s="24" t="n">
         <v>71</v>
       </c>
-      <c r="H42" t="inlineStr">
+      <c r="H42" s="24" t="inlineStr">
         <is>
           <t>אנגלית</t>
         </is>
       </c>
-      <c r="I42" t="inlineStr">
+      <c r="I42" s="24" t="inlineStr">
         <is>
           <t>תרגיל</t>
         </is>
       </c>
-      <c r="J42" t="inlineStr">
+      <c r="J42" s="24" t="inlineStr">
         <is>
           <t>גומיית רצועה ארוכה</t>
         </is>
       </c>
-      <c r="K42" t="inlineStr">
+      <c r="K42" s="24" t="inlineStr">
         <is>
           <t>מתחילים</t>
         </is>
       </c>
-      <c r="L42" t="inlineStr">
+      <c r="L42" s="24" t="inlineStr">
         <is>
           <t>חיזוק</t>
         </is>
       </c>
-      <c r="M42" t="inlineStr">
+      <c r="M42" s="24" t="inlineStr">
         <is>
           <t>גוף מלא</t>
         </is>
       </c>
-      <c r="N42">
+      <c r="N42" s="24">
         <f>'מאגר מועמדים'!T42</f>
         <v/>
       </c>
-      <c r="O42" t="inlineStr">
+      <c r="O42" s="24" t="inlineStr">
         <is>
           <t>אושר לקטלוג. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל (oembed+lengthSeconds); לא נצפה תוכן במלואו.]</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" t="n">
+      <c r="A43" s="24" t="n">
         <v>42</v>
       </c>
-      <c r="B43" t="inlineStr">
+      <c r="B43" s="24" t="inlineStr">
         <is>
           <t>10 Minute Pilates Ring Workout for Inner Thighs &amp; Core | Quick, Effective &amp; Low-Impact</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
+      <c r="C43" s="24" t="inlineStr">
         <is>
           <t>The Girl With The Pilates Mat</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr">
+      <c r="D43" s="24" t="inlineStr">
         <is>
           <t>The Girl With The Pilates Mat</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr">
+      <c r="E43" s="24" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=3xNZTmlwkzk</t>
         </is>
       </c>
-      <c r="F43" t="inlineStr">
+      <c r="F43" s="24" t="inlineStr">
         <is>
           <t>לא אומת</t>
         </is>
       </c>
-      <c r="G43" t="n">
+      <c r="G43" s="24" t="n">
         <v>12</v>
       </c>
-      <c r="H43" t="inlineStr">
+      <c r="H43" s="24" t="inlineStr">
         <is>
           <t>אנגלית</t>
         </is>
       </c>
-      <c r="I43" t="inlineStr">
+      <c r="I43" s="24" t="inlineStr">
         <is>
           <t>תרגיל</t>
         </is>
       </c>
-      <c r="J43" t="inlineStr">
+      <c r="J43" s="24" t="inlineStr">
         <is>
           <t>טבעת פילאטיס (Ring)</t>
         </is>
       </c>
-      <c r="K43" t="inlineStr">
+      <c r="K43" s="24" t="inlineStr">
         <is>
           <t>מתחילים</t>
         </is>
       </c>
-      <c r="L43" t="inlineStr">
+      <c r="L43" s="24" t="inlineStr">
         <is>
           <t>חיזוק</t>
         </is>
       </c>
-      <c r="M43" t="inlineStr">
+      <c r="M43" s="24" t="inlineStr">
         <is>
           <t>ישבן ורגליים / בטן וליבה</t>
         </is>
       </c>
-      <c r="N43">
+      <c r="N43" s="24">
         <f>'מאגר מועמדים'!T43</f>
         <v/>
       </c>
-      <c r="O43" t="inlineStr">
+      <c r="O43" s="24" t="inlineStr">
         <is>
           <t>אושר לקטלוג. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל (oembed+lengthSeconds); לא נצפה תוכן במלואו.]</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" t="n">
+      <c r="A44" s="24" t="n">
         <v>43</v>
       </c>
-      <c r="B44" t="inlineStr">
+      <c r="B44" s="24" t="inlineStr">
         <is>
           <t>Standing Pilates Full Body Workout with Resistance Band for Beginners | 20 Mins</t>
         </is>
       </c>
-      <c r="C44" t="inlineStr">
+      <c r="C44" s="24" t="inlineStr">
         <is>
           <t>The Girl With The Pilates Mat</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
+      <c r="D44" s="24" t="inlineStr">
         <is>
           <t>The Girl With The Pilates Mat</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr">
+      <c r="E44" s="24" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=CoouH7YSrgE</t>
         </is>
       </c>
-      <c r="F44" t="inlineStr">
+      <c r="F44" s="24" t="inlineStr">
         <is>
           <t>לא אומת</t>
         </is>
       </c>
-      <c r="G44" t="n">
+      <c r="G44" s="24" t="n">
         <v>19</v>
       </c>
-      <c r="H44" t="inlineStr">
+      <c r="H44" s="24" t="inlineStr">
         <is>
           <t>אנגלית</t>
         </is>
       </c>
-      <c r="I44" t="inlineStr">
+      <c r="I44" s="24" t="inlineStr">
         <is>
           <t>תרגיל</t>
         </is>
       </c>
-      <c r="J44" t="inlineStr">
+      <c r="J44" s="24" t="inlineStr">
         <is>
           <t>גומיית רצועה ארוכה</t>
         </is>
       </c>
-      <c r="K44" t="inlineStr">
+      <c r="K44" s="24" t="inlineStr">
         <is>
           <t>מתחילים</t>
         </is>
       </c>
-      <c r="L44" t="inlineStr">
+      <c r="L44" s="24" t="inlineStr">
         <is>
           <t>חיזוק</t>
         </is>
       </c>
-      <c r="M44" t="inlineStr">
+      <c r="M44" s="24" t="inlineStr">
         <is>
           <t>גוף מלא</t>
         </is>
       </c>
-      <c r="N44">
+      <c r="N44" s="24">
         <f>'מאגר מועמדים'!T44</f>
         <v/>
       </c>
-      <c r="O44" t="inlineStr">
+      <c r="O44" s="24" t="inlineStr">
         <is>
           <t>אושר לקטלוג. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל (oembed+lengthSeconds); לא נצפה תוכן במלואו.]</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" t="n">
+      <c r="A45" s="24" t="n">
         <v>44</v>
       </c>
-      <c r="B45" t="inlineStr">
+      <c r="B45" s="24" t="inlineStr">
         <is>
           <t>Standing Pilates Ring Workout to Tone Arms, Back and Shoulders After 40</t>
         </is>
       </c>
-      <c r="C45" t="inlineStr">
+      <c r="C45" s="24" t="inlineStr">
         <is>
           <t>The Girl With The Pilates Mat</t>
         </is>
       </c>
-      <c r="D45" t="inlineStr">
+      <c r="D45" s="24" t="inlineStr">
         <is>
           <t>The Girl With The Pilates Mat</t>
         </is>
       </c>
-      <c r="E45" t="inlineStr">
+      <c r="E45" s="24" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=ZxLJ8jbnURc</t>
         </is>
       </c>
-      <c r="F45" t="inlineStr">
+      <c r="F45" s="24" t="inlineStr">
         <is>
           <t>לא אומת</t>
         </is>
       </c>
-      <c r="G45" t="n">
+      <c r="G45" s="24" t="n">
         <v>15</v>
       </c>
-      <c r="H45" t="inlineStr">
+      <c r="H45" s="24" t="inlineStr">
         <is>
           <t>אנגלית</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr">
+      <c r="I45" s="24" t="inlineStr">
         <is>
           <t>תרגיל</t>
         </is>
       </c>
-      <c r="J45" t="inlineStr">
+      <c r="J45" s="24" t="inlineStr">
         <is>
           <t>טבעת פילאטיס (Ring)</t>
         </is>
       </c>
-      <c r="K45" t="inlineStr">
+      <c r="K45" s="24" t="inlineStr">
         <is>
           <t>מתחילים</t>
         </is>
       </c>
-      <c r="L45" t="inlineStr">
+      <c r="L45" s="24" t="inlineStr">
         <is>
           <t>חיזוק</t>
         </is>
       </c>
-      <c r="M45" t="inlineStr">
+      <c r="M45" s="24" t="inlineStr">
         <is>
           <t>כתפיים וזרועות / גב ויציבה</t>
         </is>
       </c>
-      <c r="N45">
+      <c r="N45" s="24">
         <f>'מאגר מועמדים'!T45</f>
         <v/>
       </c>
-      <c r="O45" t="inlineStr">
+      <c r="O45" s="24" t="inlineStr">
         <is>
           <t>אושר לקטלוג. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל (oembed+lengthSeconds); לא נצפה תוכן במלואו.]</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" t="n">
+      <c r="A46" s="24" t="n">
         <v>45</v>
       </c>
-      <c r="B46" t="inlineStr">
+      <c r="B46" s="24" t="inlineStr">
         <is>
           <t>15 Min Upper Body Resistance Band Workout for Strong Back, Arms and Shoulders | Pilates Arm Workout</t>
         </is>
       </c>
-      <c r="C46" t="inlineStr">
+      <c r="C46" s="24" t="inlineStr">
         <is>
           <t>The Girl With The Pilates Mat</t>
         </is>
       </c>
-      <c r="D46" t="inlineStr">
+      <c r="D46" s="24" t="inlineStr">
         <is>
           <t>The Girl With The Pilates Mat</t>
         </is>
       </c>
-      <c r="E46" t="inlineStr">
+      <c r="E46" s="24" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=JdO0B4MkhTM</t>
         </is>
       </c>
-      <c r="F46" t="inlineStr">
+      <c r="F46" s="24" t="inlineStr">
         <is>
           <t>לא אומת</t>
         </is>
       </c>
-      <c r="G46" t="n">
+      <c r="G46" s="24" t="n">
         <v>16</v>
       </c>
-      <c r="H46" t="inlineStr">
+      <c r="H46" s="24" t="inlineStr">
         <is>
           <t>אנגלית</t>
         </is>
       </c>
-      <c r="I46" t="inlineStr">
+      <c r="I46" s="24" t="inlineStr">
         <is>
           <t>תרגיל</t>
         </is>
       </c>
-      <c r="J46" t="inlineStr">
+      <c r="J46" s="24" t="inlineStr">
         <is>
           <t>גומיית רצועה ארוכה</t>
         </is>
       </c>
-      <c r="K46" t="inlineStr">
+      <c r="K46" s="24" t="inlineStr">
         <is>
           <t>מתחילים</t>
         </is>
       </c>
-      <c r="L46" t="inlineStr">
+      <c r="L46" s="24" t="inlineStr">
         <is>
           <t>חיזוק</t>
         </is>
       </c>
-      <c r="M46" t="inlineStr">
+      <c r="M46" s="24" t="inlineStr">
         <is>
           <t>כתפיים וזרועות / גב ויציבה</t>
         </is>
       </c>
-      <c r="N46">
+      <c r="N46" s="24">
         <f>'מאגר מועמדים'!T46</f>
         <v/>
       </c>
-      <c r="O46" t="inlineStr">
+      <c r="O46" s="24" t="inlineStr">
         <is>
           <t>אושר לקטלוג. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל (oembed+lengthSeconds); לא נצפה תוכן במלואו.]</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" t="n">
+      <c r="A47" s="24" t="n">
         <v>46</v>
       </c>
-      <c r="B47" t="inlineStr">
+      <c r="B47" s="24" t="inlineStr">
         <is>
           <t>Resistance Band Pilates Workout 25 Min</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C47" s="24" t="inlineStr">
         <is>
           <t>The Girl With The Pilates Mat</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="D47" s="24" t="inlineStr">
         <is>
           <t>The Girl With The Pilates Mat</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
+      <c r="E47" s="24" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=bpkB4E4aNNw</t>
         </is>
       </c>
-      <c r="F47" t="inlineStr">
+      <c r="F47" s="24" t="inlineStr">
         <is>
           <t>לא אומת</t>
         </is>
       </c>
-      <c r="G47" t="n">
+      <c r="G47" s="24" t="n">
         <v>53</v>
       </c>
-      <c r="H47" t="inlineStr">
+      <c r="H47" s="24" t="inlineStr">
         <is>
           <t>אנגלית</t>
         </is>
       </c>
-      <c r="I47" t="inlineStr">
+      <c r="I47" s="24" t="inlineStr">
         <is>
           <t>תרגיל</t>
         </is>
       </c>
-      <c r="J47" t="inlineStr">
+      <c r="J47" s="24" t="inlineStr">
         <is>
           <t>גומיית רצועה ארוכה</t>
         </is>
       </c>
-      <c r="K47" t="inlineStr">
+      <c r="K47" s="24" t="inlineStr">
         <is>
           <t>מתחילים</t>
         </is>
       </c>
-      <c r="L47" t="inlineStr">
+      <c r="L47" s="24" t="inlineStr">
         <is>
           <t>חיזוק</t>
         </is>
       </c>
-      <c r="M47" t="inlineStr">
+      <c r="M47" s="24" t="inlineStr">
         <is>
           <t>גוף מלא</t>
         </is>
       </c>
-      <c r="N47">
+      <c r="N47" s="24">
         <f>'מאגר מועמדים'!T47</f>
         <v/>
       </c>
-      <c r="O47" t="inlineStr">
+      <c r="O47" s="24" t="inlineStr">
         <is>
           <t>אושר לקטלוג. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל (oembed+lengthSeconds); לא נצפה תוכן במלואו.]</t>
         </is>
@@ -11873,7 +11873,7 @@
       </c>
       <c r="C3" s="39" t="inlineStr">
         <is>
-          <t>https://www.youtube.com/@JessicaValantPilates</t>
+          <t>https://www.youtube.com/@Jessicasvalant</t>
         </is>
       </c>
       <c r="D3" s="33" t="inlineStr">
@@ -11883,19 +11883,19 @@
       </c>
       <c r="E3" s="34" t="inlineStr">
         <is>
-          <t>טכניקה ובטיחות, שיקום</t>
+          <t>טכניקה ובטיחות, שיקום, בריאות האישה</t>
         </is>
       </c>
       <c r="F3" s="34" t="inlineStr">
         <is>
-          <t>פיזיותרפיסטית מוסמכת, 16+ שנה</t>
+          <t>פיזיותרפיסטית מוסמכת, 25+ שנות ניסיון</t>
         </is>
       </c>
       <c r="G3" s="33" t="n"/>
       <c r="H3" s="35" t="n"/>
       <c r="I3" s="34" t="inlineStr">
         <is>
-          <t>דגש בטיחותי חזק - מתאים לקהל מבוגרים/שיקום</t>
+          <t>דגש בטיחותי חזק - מתאים לקהל מבוגרים/שיקום [עודכן ע"י Claude, 30.08.2026: הקישור המקורי (@JessicaValantPilates) שבור (404) - תוקן לכתובת האמיתית @Jessicasvalant, שאומתה כבר קודם מול הסרטונים שנוספו בפועל. אומת: 1.15M מנויים, 692 סרטונים, פעילה מ-09/2013.]</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Document mixed-content channel policy, approve Move With Nicole
Clarified that a channel with substantial Pilates content alongside
yoga/general fitness can be approved if it meets the other criteria -
selection happens per-video, not by channel exclusivity. Added as a
formal criterion in the core-principles sheet and approved "Move
With Nicole" accordingly (credentials verified word-for-word against
her channel bio), with a caveat that her claimed band/ring equipment
content wasn't confirmed in recent uploads.
</commit_message>
<xml_diff>
--- a/YR1/pilates/data/מטריצת_כיסוי_קטלוג_פילאטיס_v5.xlsx
+++ b/YR1/pilates/data/מטריצת_כיסוי_קטלוג_פילאטיס_v5.xlsx
@@ -600,7 +600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:A54"/>
+  <dimension ref="A1:A55"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6171875" defaultRowHeight="13.5" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="115" customWidth="1" style="24" min="1" max="1"/>
@@ -958,6 +958,13 @@
       <c r="A54" s="24" t="inlineStr">
         <is>
           <t>• 30.08.2026: עברתי על סרטוני הערוץ "The Girl With The Pilates Mat" לבקשת המשתמש - נוספו 12 סרטונים חדשים (#35-46). סגרו לגמרי: #7,#13,#25,#26 (הושלמו); הרחיבו משמעותית: #4,#24,#28 (חלקי); #29 עבר את היעד בהרבה (מותר לפי הנחיית המשתמש). 2 סרטונים (בינוני/כדור-קטן-בינוני) לא תאמו משבצת קיימת - נוספו כתוכן בונוס.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>• החלטת מדיניות, 30.08.2026 (לבקשת המשתמש): ערוץ עם כמות משמעותית של תוכן פילאטיס יחד עם תוכן יוגה יכול להיות מאושר, בתנאי שעומד בשאר הקריטריונים - הבחירה בפועל תמיד תהיה לפי סרטון ספציפי (פילאטיס בלבד), לא לפי בלעדיות תוכן הערוץ. נוסף גם כקריטריון מפורש בגיליון "עקרונות ליבה". בעקבות זה, "Move With Nicole" (שנבדק בסבב הקודם והוכשרה שלה אומתה, אך סומן כמעורב יוגה) עודכן ל"מאושר".</t>
         </is>
       </c>
     </row>
@@ -7905,7 +7912,7 @@
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation sqref="D2:D41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
-      <formula1>'ערוצים מאושרים'!$B$2:$B$21</formula1>
+      <formula1>'ערוצים מאושרים'!$B$2:$B$22</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -11348,7 +11355,7 @@
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation sqref="D2:D41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
-      <formula1>'ערוצים מאושרים'!$B$2:$B$21</formula1>
+      <formula1>'ערוצים מאושרים'!$B$2:$B$22</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -11377,7 +11384,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:K22"/>
+  <dimension ref="A1:K23"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6171875" defaultRowHeight="13.5" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="20" customWidth="1" style="24" min="1" max="1"/>
@@ -11727,6 +11734,23 @@
       <c r="D22" s="34" t="inlineStr">
         <is>
           <t>למחוק אם מתקיים</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>מקור ואמינות</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ערוץ עם תוכן פילאטיס משמעותי (לא בהכרח בלעדי) - שילוב יוגה/כושר כללי לצידו מקובל</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>הובהר ע"י המשתמש, 30.08.2026 - נבחר לפי הסרטון הספציפי שנוסף לקטלוג, לא לפי בלעדיות תוכן הערוץ.</t>
         </is>
       </c>
     </row>
@@ -11758,7 +11782,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:K21"/>
+  <dimension ref="A1:K22"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6171875" defaultRowHeight="13.5" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="6" customWidth="1" style="24" min="1" max="1"/>
@@ -12554,6 +12578,43 @@
       <c r="I21" s="24" t="inlineStr">
         <is>
           <t>נוסף ע"י Claude, 30.08.2026 - אותר דרך סרטון ספציפי שביקש המשתמש. 114K מנויים, 1,118 סרטונים - עמותה רפואית מוכרת ומבוססת (לא מדריך/ה עצמאי/ת), רמת אמינות גבוהה מאוד למרות שאינה "ערוץ פילאטיס" במובן הרגיל - תוכן פעילות גופנית/שיקום לב מבוסס-בטיחות.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Move With Nicole</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/@MoveWithNicole</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>מאושר</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>פילאטיס (מזרן/רפורמר) ויוגה, כולל תוכן טרום/אחרי לידה</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>Certified Pilates &amp; Reformer Instructor, Certified Yoga Instructor (RYT 500), Pre/Postnatal Pilates &amp; Coaching Specialist, Personal Trainer</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>נבדק ע"י Claude, 30.08.2026: 6.16M מנויים (בפועל גבוה משמעותית ממה שדווח בתחילה - 3.5M), 246 סרטונים, פעילה מ-03/2019. הכשרה אומתה מילה-במילה מול ביו הערוץ עצמו. הערוץ משלב יוגה לצד פילאטיס - הוחלט (ע"י המשתמש) שזה מקובל, הבחירה תהיה לפי סרטון ולא לפי בלעדיות הערוץ. הסתייגות: 15 הסרטונים האחרונים שנבדקו כולם "ללא ציוד" - הטענה על תוכן רינג/משקולות/גומיות לא אומתה בפועל, יש לבדוק פר-סרטון לפני הוספה.</t>
         </is>
       </c>
     </row>
@@ -13604,7 +13665,7 @@
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation sqref="E2:E14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
-      <formula1>'ערוצים מאושרים'!$B$2:$B$21</formula1>
+      <formula1>'ערוצים מאושרים'!$B$2:$B$22</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Approve IsaWelly Pilates after verifying STOTT certification
Checked the press page the user linked plus a web search: her own
channel bio is blank, but STOTT Pilates certification and
significant press coverage (Elle Australia, PopSugar, Grazia, Vogue
UK, Adidas, Sweaty Betty) are independently confirmed. Resolves the
earlier credential concern; the equipment-content claim still needs
per-video verification.
</commit_message>
<xml_diff>
--- a/YR1/pilates/data/מטריצת_כיסוי_קטלוג_פילאטיס_v5.xlsx
+++ b/YR1/pilates/data/מטריצת_כיסוי_קטלוג_פילאטיס_v5.xlsx
@@ -600,7 +600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:A55"/>
+  <dimension ref="A1:A56"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6171875" defaultRowHeight="13.5" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="115" customWidth="1" style="24" min="1" max="1"/>
@@ -962,9 +962,16 @@
       </c>
     </row>
     <row r="55">
-      <c r="A55" t="inlineStr">
+      <c r="A55" s="24" t="inlineStr">
         <is>
           <t>• החלטת מדיניות, 30.08.2026 (לבקשת המשתמש): ערוץ עם כמות משמעותית של תוכן פילאטיס יחד עם תוכן יוגה יכול להיות מאושר, בתנאי שעומד בשאר הקריטריונים - הבחירה בפועל תמיד תהיה לפי סרטון ספציפי (פילאטיס בלבד), לא לפי בלעדיות תוכן הערוץ. נוסף גם כקריטריון מפורש בגיליון "עקרונות ליבה". בעקבות זה, "Move With Nicole" (שנבדק בסבב הקודם והוכשרה שלה אומתה, אך סומן כמעורב יוגה) עודכן ל"מאושר".</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>• 30.08.2026: המשתמש ביקש לבדוק https://isawellypilates.com/press/ ולחפש ברשת מידע על הכשרתה של IsaWelly Pilates (שסומנה קודם כלא-מאומתת, ביו הערוץ ריק). אומת חיצונית: מוסמכת STOTT Pilates + כיסוי תקשורתי משמעותי (Elle Australia, PopSugar, Grazia, Vogue UK, Adidas, Sweaty Betty). עודכנה ל"מאושר".</t>
         </is>
       </c>
     </row>
@@ -7912,7 +7919,7 @@
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation sqref="D2:D41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
-      <formula1>'ערוצים מאושרים'!$B$2:$B$22</formula1>
+      <formula1>'ערוצים מאושרים'!$B$2:$B$23</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -11355,7 +11362,7 @@
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation sqref="D2:D41" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
-      <formula1>'ערוצים מאושרים'!$B$2:$B$22</formula1>
+      <formula1>'ערוצים מאושרים'!$B$2:$B$23</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -11738,17 +11745,17 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="24" t="inlineStr">
         <is>
           <t>מקור ואמינות</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="24" t="inlineStr">
         <is>
           <t>ערוץ עם תוכן פילאטיס משמעותי (לא בהכרח בלעדי) - שילוב יוגה/כושר כללי לצידו מקובל</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" s="24" t="inlineStr">
         <is>
           <t>הובהר ע"י המשתמש, 30.08.2026 - נבחר לפי הסרטון הספציפי שנוסף לקטלוג, לא לפי בלעדיות תוכן הערוץ.</t>
         </is>
@@ -11782,7 +11789,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:K22"/>
+  <dimension ref="A1:K23"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6171875" defaultRowHeight="13.5" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="6" customWidth="1" style="24" min="1" max="1"/>
@@ -12582,39 +12589,80 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="n">
+      <c r="A22" s="24" t="n">
         <v>21</v>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B22" s="24" t="inlineStr">
         <is>
           <t>Move With Nicole</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C22" s="24" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@MoveWithNicole</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D22" s="24" t="inlineStr">
         <is>
           <t>מאושר</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E22" s="24" t="inlineStr">
         <is>
           <t>פילאטיס (מזרן/רפורמר) ויוגה, כולל תוכן טרום/אחרי לידה</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="F22" s="24" t="inlineStr">
         <is>
           <t>Certified Pilates &amp; Reformer Instructor, Certified Yoga Instructor (RYT 500), Pre/Postnatal Pilates &amp; Coaching Specialist, Personal Trainer</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
-      <c r="I22" t="inlineStr">
+      <c r="G22" s="24" t="inlineStr"/>
+      <c r="H22" s="24" t="inlineStr"/>
+      <c r="I22" s="24" t="inlineStr">
         <is>
           <t>נבדק ע"י Claude, 30.08.2026: 6.16M מנויים (בפועל גבוה משמעותית ממה שדווח בתחילה - 3.5M), 246 סרטונים, פעילה מ-03/2019. הכשרה אומתה מילה-במילה מול ביו הערוץ עצמו. הערוץ משלב יוגה לצד פילאטיס - הוחלט (ע"י המשתמש) שזה מקובל, הבחירה תהיה לפי סרטון ולא לפי בלעדיות הערוץ. הסתייגות: 15 הסרטונים האחרונים שנבדקו כולם "ללא ציוד" - הטענה על תוכן רינג/משקולות/גומיות לא אומתה בפועל, יש לבדוק פר-סרטון לפני הוספה.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>IsaWelly Pilates</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/@IsaWellyPilates</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>מאושר</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>פילאטיס מזרן, תוכניות מובנות (The Pilates School, RESILIENT), חיזוק כללי</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>מוסמכת STOTT Pilates, 20+ שנות ניסיון, רקדנית מקצועית לשעבר (מעל עשור)</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>https://isawellypilates.com/press/</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>נבדק ע"י Claude, 30.08.2026, לבקשת המשתמש - נבדק https://isawellypilates.com/press/ + חיפוש רשת נוסף: הביו של הערוץ עצמו ריק/לא כולל הסמכה, אך אומת חיצונית שהיא מוסמכת STOTT Pilates (גוף הסמכה מוכר), 20 שנות ניסיון עם פילאטיס ורקע כרקדנית מקצועית. כיסוי תקשורתי משמעותי מאמת אמינות: Elle Australia ("10 Best Pilates Teachers on YouTube"), PopSugar, Grazia, Vogue UK, שיתופי פעולה עם Adidas ו-Sweaty Betty. 515K מנויים, 251 סרטונים, פעילה מ-05/2016. הסתייגות שנותרה: 15 הסרטונים האחרונים שנבדקו קודם היו כולם "ללא ציוד" - הטענה על דגש חזק על גומיות/כדורים לא אומתה בפועל, יש לבדוק פר-סרטון.</t>
         </is>
       </c>
     </row>
@@ -13665,7 +13713,7 @@
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation sqref="E2:E14" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list" errorStyle="stop" operator="between">
-      <formula1>'ערוצים מאושרים'!$B$2:$B$22</formula1>
+      <formula1>'ערוצים מאושרים'!$B$2:$B$23</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Approve 4 reviewed channels, add 28 videos across many topics
Finalized approval for Jessica Valant Pilates, Move With Nicole,
IsaWelly Pilates, and Flow with Mira. Cataloged 20 short exercise
videos spanning many topics (shoulder/hip/back rehab, core, inner
thigh, balance, full body) and 8 lesson-length videos (30+ minutes,
verified against real runtime) from their channels, adding depth
beyond target where the matrix cell was already met, per instruction.

Several titles significantly misrepresented actual duration in both
directions (e.g. "10 Min" videos running 40+ minutes, and "45 MIN"
videos running under 22) - classification used verified runtime, not
the title claim.
</commit_message>
<xml_diff>
--- a/YR1/pilates/data/מטריצת_כיסוי_קטלוג_פילאטיס_v5.xlsx
+++ b/YR1/pilates/data/מטריצת_כיסוי_קטלוג_פילאטיס_v5.xlsx
@@ -600,7 +600,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:A56"/>
+  <dimension ref="A1:A57"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6171875" defaultRowHeight="13.5" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="115" customWidth="1" style="24" min="1" max="1"/>
@@ -969,9 +969,16 @@
       </c>
     </row>
     <row r="56">
-      <c r="A56" t="inlineStr">
+      <c r="A56" s="24" t="inlineStr">
         <is>
           <t>• 30.08.2026: המשתמש ביקש לבדוק https://isawellypilates.com/press/ ולחפש ברשת מידע על הכשרתה של IsaWelly Pilates (שסומנה קודם כלא-מאומתת, ביו הערוץ ריק). אומת חיצונית: מוסמכת STOTT Pilates + כיסוי תקשורתי משמעותי (Elle Australia, PopSugar, Grazia, Vogue UK, Adidas, Sweaty Betty). עודכנה ל"מאושר".</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>• 30.08.2026: אושרו סופית 4 הערוצים שנבדקו (Jessica Valant Pilates, Move With Nicole, IsaWelly Pilates, Flow with Mira) - כולם "מאושר". קוטלגו מהם 28 סרטונים (20 תרגילים קצרים במגוון נושאים + 8 שיעורים מעל חצי שעה בפועל), לבקשת המשתמש - כולל תוספת למשבצות שכבר מעל היעד. גילוי חשוב: כמה כותרות הבטיחו משך קצר ("10 דקות") אך המשך האמיתי היה הרבה יותר ארוך (עד 42 דקות) ולהיפך ("30/45 דקות" שהתבררו כ-12-22 דקות בפועל) - הסיווג תרגיל/שיעור נקבע לפי המשך האמיתי שאומת, לא לפי הכותרת.</t>
         </is>
       </c>
     </row>
@@ -1110,7 +1117,7 @@
         <v>2</v>
       </c>
       <c r="J2" s="35" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="K2" s="33">
         <f>IF(J2=0,"חסר",IF(J2&lt;I2,"בתהליך","הושלם"))</f>
@@ -1161,7 +1168,7 @@
         <v>1</v>
       </c>
       <c r="J3" s="35" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K3" s="33">
         <f>IF(J3=0,"חסר",IF(J3&lt;I3,"בתהליך","הושלם"))</f>
@@ -1518,7 +1525,7 @@
         <v>2</v>
       </c>
       <c r="J10" s="35" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K10" s="33">
         <f>IF(J10=0,"חסר",IF(J10&lt;I10,"בתהליך","הושלם"))</f>
@@ -1773,7 +1780,7 @@
         <v>4</v>
       </c>
       <c r="J15" s="35" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="K15" s="33">
         <f>IF(J15=0,"חסר",IF(J15&lt;I15,"בתהליך","הושלם"))</f>
@@ -2193,7 +2200,7 @@
         <v>2</v>
       </c>
       <c r="J23" s="35" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K23" s="33">
         <f>IF(J26=0,"חסר",IF(J26&lt;I26,"בתהליך","הושלם"))</f>
@@ -2244,7 +2251,7 @@
         <v>1</v>
       </c>
       <c r="J24" s="35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K24" s="33">
         <f>IF(J27=0,"חסר",IF(J27&lt;I27,"בתהליך","הושלם"))</f>
@@ -2448,7 +2455,7 @@
         <v>2</v>
       </c>
       <c r="J28" s="35" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="K28" s="33">
         <f>IF(J31=0,"חסר",IF(J31&lt;I31,"בתהליך","הושלם"))</f>
@@ -2743,7 +2750,7 @@
         <v>2</v>
       </c>
       <c r="F2" s="35" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G2" s="33">
         <f>IF(F2=0,"חסר",IF(F2&lt;E2,"בתהליך","הושלם"))</f>
@@ -2805,7 +2812,7 @@
         <v>1</v>
       </c>
       <c r="F4" s="35" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G4" s="33">
         <f>IF(F4=0,"חסר",IF(F4&lt;E4,"בתהליך","הושלם"))</f>
@@ -2898,7 +2905,7 @@
         <v>1</v>
       </c>
       <c r="F7" s="35" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G7" s="33">
         <f>IF(F7=0,"חסר",IF(F7&lt;E7,"בתהליך","הושלם"))</f>
@@ -3115,7 +3122,7 @@
         <v>2</v>
       </c>
       <c r="F14" s="35" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G14" s="33">
         <f>IF(F14=0,"חסר",IF(F14&lt;E14,"בתהליך","הושלם"))</f>
@@ -3417,7 +3424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:V47"/>
+  <dimension ref="A1:V75"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6171875" defaultRowHeight="13.5" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="6" customWidth="1" style="24" min="1" max="1"/>
@@ -7875,6 +7882,2638 @@
       <c r="V47" s="24" t="inlineStr">
         <is>
           <t>ערוץ מאושר (Master-level Certified Pilates Instructor). [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל (oembed+lengthSeconds); לא נצפה תוכן במלואו.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>10 Minute SHOULDER PAIN RELIEF EXERCISES - At Home</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Jessica Valant</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Jessica Valant Pilates</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=fqyaEamOyMw</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G48" t="n">
+        <v>14</v>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>ללא ציוד</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>שיקום ותנועה עדינה</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>כתפיים וזרועות</t>
+        </is>
+      </c>
+      <c r="N48" t="n">
+        <v>4</v>
+      </c>
+      <c r="O48" t="n">
+        <v>4</v>
+      </c>
+      <c r="P48" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q48" t="n">
+        <v>5</v>
+      </c>
+      <c r="R48" t="n">
+        <v>4</v>
+      </c>
+      <c r="S48" t="n">
+        <v>5</v>
+      </c>
+      <c r="T48" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="U48" t="inlineStr">
+        <is>
+          <t>לכלול בקטלוג</t>
+        </is>
+      </c>
+      <c r="V48" t="inlineStr">
+        <is>
+          <t>ערוץ מאושר. תרגילים להקלה על כאבי כתפיים, ללא ציוד, מפיזיותרפיסטית ומדריכת פילאטיס מוסמכת. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>HYSTERECTOMY WORKOUT - 10 Min Exercises After Hysterectomy</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Jessica Valant</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Jessica Valant Pilates</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=D2TK7OLH0Pg</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G49" t="n">
+        <v>12</v>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>ללא ציוד</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>שיקום ותנועה עדינה</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>בטן וליבה</t>
+        </is>
+      </c>
+      <c r="N49" t="n">
+        <v>4</v>
+      </c>
+      <c r="O49" t="n">
+        <v>4</v>
+      </c>
+      <c r="P49" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q49" t="n">
+        <v>5</v>
+      </c>
+      <c r="R49" t="n">
+        <v>4</v>
+      </c>
+      <c r="S49" t="n">
+        <v>5</v>
+      </c>
+      <c r="T49" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="U49" t="inlineStr">
+        <is>
+          <t>לכלול בקטלוג</t>
+        </is>
+      </c>
+      <c r="V49" t="inlineStr">
+        <is>
+          <t>ערוץ מאושר. תרגילים עדינים לבטן אחרי כריתת רחם, ללא ציוד. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>LYMPHATIC DRAINAGE EXERCISES- 10 Minute Lymphatic Workout at Home</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Jessica Valant</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Jessica Valant Pilates</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=IuSZW_uxDEo</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G50" t="n">
+        <v>16</v>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>ללא ציוד</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>שיקום ותנועה עדינה</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>גוף מלא</t>
+        </is>
+      </c>
+      <c r="N50" t="n">
+        <v>4</v>
+      </c>
+      <c r="O50" t="n">
+        <v>4</v>
+      </c>
+      <c r="P50" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q50" t="n">
+        <v>5</v>
+      </c>
+      <c r="R50" t="n">
+        <v>4</v>
+      </c>
+      <c r="S50" t="n">
+        <v>5</v>
+      </c>
+      <c r="T50" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="U50" t="inlineStr">
+        <is>
+          <t>לכלול בקטלוג</t>
+        </is>
+      </c>
+      <c r="V50" t="inlineStr">
+        <is>
+          <t>ערוץ מאושר. תרגילי ניקוז לימפתי עדינים לגוף מלא, ללא ציוד. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>DISC HERNIATION EXERCISES - Lower Back Pain Exercises at Home</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Jessica Valant</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Jessica Valant Pilates</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=xHgSA1zEcQ0</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G51" t="n">
+        <v>13</v>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>ללא ציוד</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>שיקום ותנועה עדינה</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>גב ויציבה</t>
+        </is>
+      </c>
+      <c r="N51" t="n">
+        <v>4</v>
+      </c>
+      <c r="O51" t="n">
+        <v>4</v>
+      </c>
+      <c r="P51" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q51" t="n">
+        <v>5</v>
+      </c>
+      <c r="R51" t="n">
+        <v>4</v>
+      </c>
+      <c r="S51" t="n">
+        <v>5</v>
+      </c>
+      <c r="T51" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="U51" t="inlineStr">
+        <is>
+          <t>לכלול בקטלוג</t>
+        </is>
+      </c>
+      <c r="V51" t="inlineStr">
+        <is>
+          <t>ערוץ מאושר. תרגילים לכאבי גב תחתון עקב בקע דיסק, ללא ציוד. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>10 Minute INNER THIGH WORKOUT</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Jessica Valant</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Jessica Valant Pilates</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=iuckX9cU0tM</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G52" t="n">
+        <v>12</v>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>ללא ציוד</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>ישבן ורגליים</t>
+        </is>
+      </c>
+      <c r="N52" t="n">
+        <v>4</v>
+      </c>
+      <c r="O52" t="n">
+        <v>4</v>
+      </c>
+      <c r="P52" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q52" t="n">
+        <v>5</v>
+      </c>
+      <c r="R52" t="n">
+        <v>4</v>
+      </c>
+      <c r="S52" t="n">
+        <v>5</v>
+      </c>
+      <c r="T52" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="U52" t="inlineStr">
+        <is>
+          <t>לכלול בקטלוג</t>
+        </is>
+      </c>
+      <c r="V52" t="inlineStr">
+        <is>
+          <t>ערוץ מאושר. תרגול ממוקד לירך פנימית, ללא ציוד. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>HIP EXERCISES - Hip Impingement &amp; Hip Labral Tear Exercises</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Jessica Valant</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Jessica Valant Pilates</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=PKWrjZkKgCo</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G53" t="n">
+        <v>12</v>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>ללא ציוד</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>שיקום ותנועה עדינה</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>ישבן ורגליים</t>
+        </is>
+      </c>
+      <c r="N53" t="n">
+        <v>4</v>
+      </c>
+      <c r="O53" t="n">
+        <v>4</v>
+      </c>
+      <c r="P53" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q53" t="n">
+        <v>5</v>
+      </c>
+      <c r="R53" t="n">
+        <v>4</v>
+      </c>
+      <c r="S53" t="n">
+        <v>5</v>
+      </c>
+      <c r="T53" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="U53" t="inlineStr">
+        <is>
+          <t>לכלול בקטלוג</t>
+        </is>
+      </c>
+      <c r="V53" t="inlineStr">
+        <is>
+          <t>ערוץ מאושר. תרגילים למפרק ירך (התנגשות ירך/קרע שפה מפרקית), ללא ציוד. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>10 Minute PILATES CORE WORKOUT - Beginner Friendly!</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Jessica Valant</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Jessica Valant Pilates</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=O3RGbWPqqf8</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G54" t="n">
+        <v>11</v>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>ללא ציוד</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>בטן וליבה</t>
+        </is>
+      </c>
+      <c r="N54" t="n">
+        <v>4</v>
+      </c>
+      <c r="O54" t="n">
+        <v>4</v>
+      </c>
+      <c r="P54" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q54" t="n">
+        <v>5</v>
+      </c>
+      <c r="R54" t="n">
+        <v>4</v>
+      </c>
+      <c r="S54" t="n">
+        <v>5</v>
+      </c>
+      <c r="T54" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="U54" t="inlineStr">
+        <is>
+          <t>לכלול בקטלוג</t>
+        </is>
+      </c>
+      <c r="V54" t="inlineStr">
+        <is>
+          <t>ערוץ מאושר. תרגול ליבה למתחילים, ללא ציוד. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>10 MIN FULL BODY WORKOUT - No Equipment!</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Jessica Valant</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Jessica Valant Pilates</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=-5FAtYJBZ1A</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G55" t="n">
+        <v>12</v>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>ללא ציוד</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>גוף מלא</t>
+        </is>
+      </c>
+      <c r="N55" t="n">
+        <v>4</v>
+      </c>
+      <c r="O55" t="n">
+        <v>4</v>
+      </c>
+      <c r="P55" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q55" t="n">
+        <v>5</v>
+      </c>
+      <c r="R55" t="n">
+        <v>4</v>
+      </c>
+      <c r="S55" t="n">
+        <v>5</v>
+      </c>
+      <c r="T55" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="U55" t="inlineStr">
+        <is>
+          <t>לכלול בקטלוג</t>
+        </is>
+      </c>
+      <c r="V55" t="inlineStr">
+        <is>
+          <t>ערוץ מאושר. אימון גוף מלא קצר ללא ציוד, למתחילים. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>10 Min STRETCHES AFTER RUNNING</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Jessica Valant</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Jessica Valant Pilates</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=rWz2vOuK8Oo</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G56" t="n">
+        <v>40</v>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>שיעור</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>ללא ציוד</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>גמישות ומתיחות</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>ישבן ורגליים</t>
+        </is>
+      </c>
+      <c r="N56" t="n">
+        <v>4</v>
+      </c>
+      <c r="O56" t="n">
+        <v>4</v>
+      </c>
+      <c r="P56" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q56" t="n">
+        <v>5</v>
+      </c>
+      <c r="R56" t="n">
+        <v>4</v>
+      </c>
+      <c r="S56" t="n">
+        <v>5</v>
+      </c>
+      <c r="T56" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="U56" t="inlineStr">
+        <is>
+          <t>לכלול בקטלוג</t>
+        </is>
+      </c>
+      <c r="V56" t="inlineStr">
+        <is>
+          <t>ערוץ מאושר. שיעור מתיחות ארוך לרגליים אחרי ריצה, ללא ציוד (משך אמיתי ארוך בהרבה מהמצוין בכותרת). [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>10 Min BALANCE EXERCISES - Improve balance at home!</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Jessica Valant</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Jessica Valant Pilates</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=A89PFK8oIc8</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G57" t="n">
+        <v>37</v>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>שיעור</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>ללא ציוד</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>שיקום ותנועה עדינה</t>
+        </is>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>גוף מלא</t>
+        </is>
+      </c>
+      <c r="N57" t="n">
+        <v>4</v>
+      </c>
+      <c r="O57" t="n">
+        <v>4</v>
+      </c>
+      <c r="P57" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q57" t="n">
+        <v>5</v>
+      </c>
+      <c r="R57" t="n">
+        <v>4</v>
+      </c>
+      <c r="S57" t="n">
+        <v>5</v>
+      </c>
+      <c r="T57" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="U57" t="inlineStr">
+        <is>
+          <t>לכלול בקטלוג</t>
+        </is>
+      </c>
+      <c r="V57" t="inlineStr">
+        <is>
+          <t>ערוץ מאושר. שיעור ארוך לשיפור שיווי משקל, ללא ציוד, קצב עדין (משך אמיתי ארוך בהרבה מהמצוין בכותרת). [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>20 MIN PILATES WORKOUT || Upper Body &amp; Core (Moderate/Intermediate)</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Nicole</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Move With Nicole</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=xNCj6JnQq4Q</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G58" t="n">
+        <v>26</v>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>ללא ציוד</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>בינוני</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>כתפיים וזרועות / בטן וליבה</t>
+        </is>
+      </c>
+      <c r="N58" t="n">
+        <v>4</v>
+      </c>
+      <c r="O58" t="n">
+        <v>4</v>
+      </c>
+      <c r="P58" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q58" t="n">
+        <v>5</v>
+      </c>
+      <c r="R58" t="n">
+        <v>4</v>
+      </c>
+      <c r="S58" t="n">
+        <v>5</v>
+      </c>
+      <c r="T58" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="U58" t="inlineStr">
+        <is>
+          <t>לכלול בקטלוג</t>
+        </is>
+      </c>
+      <c r="V58" t="inlineStr">
+        <is>
+          <t>ערוץ מאושר. תרגול פלג גוף עליון וליבה ברמת ביניים, ללא ציוד. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>20 MIN PILATES CORE &amp; ABS WORKOUT || At-Home Pilates For All Levels</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Nicole</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Move With Nicole</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=_rdbS8Vko3k</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G59" t="n">
+        <v>24</v>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>ללא ציוד</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>בטן וליבה</t>
+        </is>
+      </c>
+      <c r="N59" t="n">
+        <v>4</v>
+      </c>
+      <c r="O59" t="n">
+        <v>4</v>
+      </c>
+      <c r="P59" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q59" t="n">
+        <v>5</v>
+      </c>
+      <c r="R59" t="n">
+        <v>4</v>
+      </c>
+      <c r="S59" t="n">
+        <v>5</v>
+      </c>
+      <c r="T59" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="U59" t="inlineStr">
+        <is>
+          <t>לכלול בקטלוג</t>
+        </is>
+      </c>
+      <c r="V59" t="inlineStr">
+        <is>
+          <t>ערוץ מאושר. תרגול ליבה ובטן לכל הרמות, ללא ציוד. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>35 MIN FULL BODY WORKOUT || Intermediate/Advanced Mat Pilates (No Equipment)</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Nicole</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Move With Nicole</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=1ltZQ9rJiFw</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G60" t="n">
+        <v>27</v>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>ללא ציוד</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>מתקדם</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>גוף מלא</t>
+        </is>
+      </c>
+      <c r="N60" t="n">
+        <v>4</v>
+      </c>
+      <c r="O60" t="n">
+        <v>4</v>
+      </c>
+      <c r="P60" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q60" t="n">
+        <v>5</v>
+      </c>
+      <c r="R60" t="n">
+        <v>4</v>
+      </c>
+      <c r="S60" t="n">
+        <v>5</v>
+      </c>
+      <c r="T60" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="U60" t="inlineStr">
+        <is>
+          <t>לכלול בקטלוג</t>
+        </is>
+      </c>
+      <c r="V60" t="inlineStr">
+        <is>
+          <t>ערוץ מאושר. תרגול גוף מלא מתקדם, ללא ציוד. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>10 MIN EXPRESS PILATES WORKOUT || At-Home Mat Pilates (Moderate)</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Nicole</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Move With Nicole</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=D2d7zi6ya58</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G61" t="n">
+        <v>31</v>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>שיעור</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>ללא ציוד</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>בינוני</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>גוף מלא</t>
+        </is>
+      </c>
+      <c r="N61" t="n">
+        <v>4</v>
+      </c>
+      <c r="O61" t="n">
+        <v>4</v>
+      </c>
+      <c r="P61" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q61" t="n">
+        <v>5</v>
+      </c>
+      <c r="R61" t="n">
+        <v>4</v>
+      </c>
+      <c r="S61" t="n">
+        <v>5</v>
+      </c>
+      <c r="T61" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="U61" t="inlineStr">
+        <is>
+          <t>לכלול בקטלוג</t>
+        </is>
+      </c>
+      <c r="V61" t="inlineStr">
+        <is>
+          <t>ערוץ מאושר. שיעור פילאטיס לגוף מלא ברמת ביניים, ללא ציוד (משך אמיתי ארוך יותר מהמצוין בכותרת). [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>15 MIN PILATES CORE &amp; ABS WORKOUT || Intermediate Pilates (No Equipment)</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Nicole</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Move With Nicole</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=7SU59GxGqbo</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G62" t="n">
+        <v>42</v>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>שיעור</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>ללא ציוד</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>בינוני</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>בטן וליבה</t>
+        </is>
+      </c>
+      <c r="N62" t="n">
+        <v>4</v>
+      </c>
+      <c r="O62" t="n">
+        <v>4</v>
+      </c>
+      <c r="P62" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q62" t="n">
+        <v>5</v>
+      </c>
+      <c r="R62" t="n">
+        <v>4</v>
+      </c>
+      <c r="S62" t="n">
+        <v>5</v>
+      </c>
+      <c r="T62" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="U62" t="inlineStr">
+        <is>
+          <t>לכלול בקטלוג</t>
+        </is>
+      </c>
+      <c r="V62" t="inlineStr">
+        <is>
+          <t>ערוץ מאושר. שיעור ליבה ובטן ברמת ביניים, ללא ציוד (משך אמיתי ארוך בהרבה מהמצוין בכותרת). [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>30 MIN FULL BODY WORKOUT || At-Home Pilates Ring Workout (Intermediate)</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Nicole</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Move With Nicole</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=5TzqqPJFHeQ</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G63" t="n">
+        <v>35</v>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>שיעור</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>רינג פילאטיס</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>בינוני</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>גוף מלא</t>
+        </is>
+      </c>
+      <c r="N63" t="n">
+        <v>4</v>
+      </c>
+      <c r="O63" t="n">
+        <v>4</v>
+      </c>
+      <c r="P63" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q63" t="n">
+        <v>5</v>
+      </c>
+      <c r="R63" t="n">
+        <v>4</v>
+      </c>
+      <c r="S63" t="n">
+        <v>5</v>
+      </c>
+      <c r="T63" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="U63" t="inlineStr">
+        <is>
+          <t>לכלול בקטלוג</t>
+        </is>
+      </c>
+      <c r="V63" t="inlineStr">
+        <is>
+          <t>ערוץ מאושר. שיעור פילאטיס לגוף מלא עם טבעת פילאטיס, רמת ביניים. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>50 MIN FULL BODY WORKOUT || At-Home Pilates Ring Workout (Moderate)</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Nicole</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Move With Nicole</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=toFOWvqOjDY</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G64" t="n">
+        <v>37</v>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>שיעור</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>רינג פילאטיס</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>גוף מלא</t>
+        </is>
+      </c>
+      <c r="N64" t="n">
+        <v>4</v>
+      </c>
+      <c r="O64" t="n">
+        <v>4</v>
+      </c>
+      <c r="P64" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q64" t="n">
+        <v>5</v>
+      </c>
+      <c r="R64" t="n">
+        <v>4</v>
+      </c>
+      <c r="S64" t="n">
+        <v>5</v>
+      </c>
+      <c r="T64" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="U64" t="inlineStr">
+        <is>
+          <t>לכלול בקטלוג</t>
+        </is>
+      </c>
+      <c r="V64" t="inlineStr">
+        <is>
+          <t>ערוץ מאושר. שיעור פילאטיס ארוך לגוף מלא עם טבעת פילאטיס, למתחילים. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>10MIN PILATES WORKOUT FOR STRONG CORE - QUICK AND EFFECTIVE</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>IsaWelly</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>IsaWelly Pilates</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=BIB5cc0Ah1E</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G65" t="n">
+        <v>12</v>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>ללא ציוד</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>בטן וליבה</t>
+        </is>
+      </c>
+      <c r="N65" t="n">
+        <v>4</v>
+      </c>
+      <c r="O65" t="n">
+        <v>4</v>
+      </c>
+      <c r="P65" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q65" t="n">
+        <v>5</v>
+      </c>
+      <c r="R65" t="n">
+        <v>4</v>
+      </c>
+      <c r="S65" t="n">
+        <v>5</v>
+      </c>
+      <c r="T65" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="U65" t="inlineStr">
+        <is>
+          <t>לכלול בקטלוג</t>
+        </is>
+      </c>
+      <c r="V65" t="inlineStr">
+        <is>
+          <t>ערוץ מאושר. תרגול קצר וממוקד לליבה חזקה, ללא ציוד. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>10MIN FULL -BODY PILATES WORKOUT</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>IsaWelly</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>IsaWelly Pilates</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=eCc-rkx_CXU</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G66" t="n">
+        <v>24</v>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>ללא ציוד</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>גוף מלא</t>
+        </is>
+      </c>
+      <c r="N66" t="n">
+        <v>4</v>
+      </c>
+      <c r="O66" t="n">
+        <v>4</v>
+      </c>
+      <c r="P66" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q66" t="n">
+        <v>5</v>
+      </c>
+      <c r="R66" t="n">
+        <v>4</v>
+      </c>
+      <c r="S66" t="n">
+        <v>5</v>
+      </c>
+      <c r="T66" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="U66" t="inlineStr">
+        <is>
+          <t>לכלול בקטלוג</t>
+        </is>
+      </c>
+      <c r="V66" t="inlineStr">
+        <is>
+          <t>ערוץ מאושר. תרגול לגוף מלא, ללא ציוד. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>10MIN MINDFUL MOVEMENT TO CHECK IN AND RELAX</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>IsaWelly</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>IsaWelly Pilates</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=4r4rqUGZyNE</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G67" t="n">
+        <v>21</v>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>ללא ציוד</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>שיקום ותנועה עדינה</t>
+        </is>
+      </c>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>גוף מלא</t>
+        </is>
+      </c>
+      <c r="N67" t="n">
+        <v>4</v>
+      </c>
+      <c r="O67" t="n">
+        <v>4</v>
+      </c>
+      <c r="P67" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q67" t="n">
+        <v>5</v>
+      </c>
+      <c r="R67" t="n">
+        <v>4</v>
+      </c>
+      <c r="S67" t="n">
+        <v>5</v>
+      </c>
+      <c r="T67" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="U67" t="inlineStr">
+        <is>
+          <t>לכלול בקטלוג</t>
+        </is>
+      </c>
+      <c r="V67" t="inlineStr">
+        <is>
+          <t>ערוץ מאושר. תנועה מודעת ועדינה להרפיה, ללא ציוד. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>30MIN PILATES FOR BEGINNERS</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>IsaWelly</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>IsaWelly Pilates</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=sOQ9SxEm7fc</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G68" t="n">
+        <v>12</v>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>ללא ציוד</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>גוף מלא</t>
+        </is>
+      </c>
+      <c r="N68" t="n">
+        <v>4</v>
+      </c>
+      <c r="O68" t="n">
+        <v>4</v>
+      </c>
+      <c r="P68" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q68" t="n">
+        <v>5</v>
+      </c>
+      <c r="R68" t="n">
+        <v>4</v>
+      </c>
+      <c r="S68" t="n">
+        <v>5</v>
+      </c>
+      <c r="T68" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="U68" t="inlineStr">
+        <is>
+          <t>לכלול בקטלוג</t>
+        </is>
+      </c>
+      <c r="V68" t="inlineStr">
+        <is>
+          <t>ערוץ מאושר. תרגול פילאטיס למתחילים, ללא ציוד (משך אמיתי קצר בהרבה מהמצוין בכותרת). [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>45MIN FULL BODY PILATES WORKOUT - AT HOME PILATES - GREAT FOR EVERYBODY</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>IsaWelly</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>IsaWelly Pilates</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=oKh7xDs15Kc</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G69" t="n">
+        <v>22</v>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>ללא ציוד</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>גוף מלא</t>
+        </is>
+      </c>
+      <c r="N69" t="n">
+        <v>4</v>
+      </c>
+      <c r="O69" t="n">
+        <v>4</v>
+      </c>
+      <c r="P69" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q69" t="n">
+        <v>5</v>
+      </c>
+      <c r="R69" t="n">
+        <v>4</v>
+      </c>
+      <c r="S69" t="n">
+        <v>5</v>
+      </c>
+      <c r="T69" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="U69" t="inlineStr">
+        <is>
+          <t>לכלול בקטלוג</t>
+        </is>
+      </c>
+      <c r="V69" t="inlineStr">
+        <is>
+          <t>ערוץ מאושר. תרגול גוף מלא, ללא ציוד (משך אמיתי קצר בהרבה מהמצוין בכותרת). [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>15 Min Beginner Pilates | A Real Beginner Class, Start to Finish</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Mira</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Flow with Mira</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=qk22O1Dv_2A</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G70" t="n">
+        <v>22</v>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>ללא ציוד</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>גוף מלא</t>
+        </is>
+      </c>
+      <c r="N70" t="n">
+        <v>4</v>
+      </c>
+      <c r="O70" t="n">
+        <v>4</v>
+      </c>
+      <c r="P70" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q70" t="n">
+        <v>5</v>
+      </c>
+      <c r="R70" t="n">
+        <v>4</v>
+      </c>
+      <c r="S70" t="n">
+        <v>5</v>
+      </c>
+      <c r="T70" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="U70" t="inlineStr">
+        <is>
+          <t>לכלול בקטלוג</t>
+        </is>
+      </c>
+      <c r="V70" t="inlineStr">
+        <is>
+          <t>ערוץ מאושר. שיעור אמיתי למתחילים גמורים, מתחילתו ועד סופו, ללא ציוד. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>70</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>20 Min Pilates for Core Strength &amp; Pelvic Floor | Gentle Deep Core Flow</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Mira</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Flow with Mira</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=1WDNTwAUjIw</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G71" t="n">
+        <v>13</v>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>ללא ציוד</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>שיקום ותנועה עדינה</t>
+        </is>
+      </c>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>בטן וליבה</t>
+        </is>
+      </c>
+      <c r="N71" t="n">
+        <v>4</v>
+      </c>
+      <c r="O71" t="n">
+        <v>4</v>
+      </c>
+      <c r="P71" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q71" t="n">
+        <v>5</v>
+      </c>
+      <c r="R71" t="n">
+        <v>4</v>
+      </c>
+      <c r="S71" t="n">
+        <v>5</v>
+      </c>
+      <c r="T71" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="U71" t="inlineStr">
+        <is>
+          <t>לכלול בקטלוג</t>
+        </is>
+      </c>
+      <c r="V71" t="inlineStr">
+        <is>
+          <t>ערוץ מאושר. תרגול עדין לליבה ורצפת האגן, ללא ציוד. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>71</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>20 Min Gentle Pilates for Sciatica | Relieve Nerve Pain Without Aggravating Your Back</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Mira</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Flow with Mira</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=9rerK1_8M8Y</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G72" t="n">
+        <v>25</v>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>ללא ציוד</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>שיקום ותנועה עדינה</t>
+        </is>
+      </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>ישבן ורגליים / גב ויציבה</t>
+        </is>
+      </c>
+      <c r="N72" t="n">
+        <v>4</v>
+      </c>
+      <c r="O72" t="n">
+        <v>4</v>
+      </c>
+      <c r="P72" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q72" t="n">
+        <v>5</v>
+      </c>
+      <c r="R72" t="n">
+        <v>4</v>
+      </c>
+      <c r="S72" t="n">
+        <v>5</v>
+      </c>
+      <c r="T72" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="U72" t="inlineStr">
+        <is>
+          <t>לכלול בקטלוג</t>
+        </is>
+      </c>
+      <c r="V72" t="inlineStr">
+        <is>
+          <t>ערוץ מאושר. תרגול עדין להקלה על כאב סציאטיקה בלי להעמיס על הגב, ללא ציוד. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>72</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>The 15-Min Abs &amp; Hips Workout That Doesn't Leave You Wrecked | Beginners</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Mira</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Flow with Mira</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=L7UWhrOVO3s</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G73" t="n">
+        <v>18</v>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>ללא ציוד</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t>בטן וליבה / ישבן ורגליים</t>
+        </is>
+      </c>
+      <c r="N73" t="n">
+        <v>4</v>
+      </c>
+      <c r="O73" t="n">
+        <v>4</v>
+      </c>
+      <c r="P73" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q73" t="n">
+        <v>5</v>
+      </c>
+      <c r="R73" t="n">
+        <v>4</v>
+      </c>
+      <c r="S73" t="n">
+        <v>5</v>
+      </c>
+      <c r="T73" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="U73" t="inlineStr">
+        <is>
+          <t>לכלול בקטלוג</t>
+        </is>
+      </c>
+      <c r="V73" t="inlineStr">
+        <is>
+          <t>ערוץ מאושר. תרגול בטן וירכיים למתחילים, ללא ציוד. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>73</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Pilates for Shoulder Tension | A Release Deeper Than Stretching | 20 Min</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Mira</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Flow with Mira</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Zdlqd-0pv5Q</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G74" t="n">
+        <v>32</v>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>שיעור</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>ללא ציוד</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>שיקום ותנועה עדינה</t>
+        </is>
+      </c>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t>כתפיים וזרועות</t>
+        </is>
+      </c>
+      <c r="N74" t="n">
+        <v>4</v>
+      </c>
+      <c r="O74" t="n">
+        <v>4</v>
+      </c>
+      <c r="P74" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q74" t="n">
+        <v>5</v>
+      </c>
+      <c r="R74" t="n">
+        <v>4</v>
+      </c>
+      <c r="S74" t="n">
+        <v>5</v>
+      </c>
+      <c r="T74" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="U74" t="inlineStr">
+        <is>
+          <t>לכלול בקטלוג</t>
+        </is>
+      </c>
+      <c r="V74" t="inlineStr">
+        <is>
+          <t>ערוץ מאושר. שיעור ארוך לשחרור מתח בכתפיים, ללא ציוד (משך אמיתי ארוך יותר מהמצוין בכותרת). [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>74</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Do This 30 MINUTE Full Body Pilates Workout | Beginner Pilates Workout</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Mira</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Flow with Mira</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=gOZyYIPfbVg</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G75" t="n">
+        <v>30</v>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>שיעור</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>ללא ציוד</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t>גוף מלא</t>
+        </is>
+      </c>
+      <c r="N75" t="n">
+        <v>4</v>
+      </c>
+      <c r="O75" t="n">
+        <v>4</v>
+      </c>
+      <c r="P75" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q75" t="n">
+        <v>5</v>
+      </c>
+      <c r="R75" t="n">
+        <v>4</v>
+      </c>
+      <c r="S75" t="n">
+        <v>5</v>
+      </c>
+      <c r="T75" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="U75" t="inlineStr">
+        <is>
+          <t>לכלול בקטלוג</t>
+        </is>
+      </c>
+      <c r="V75" t="inlineStr">
+        <is>
+          <t>ערוץ מאושר. שיעור פילאטיס לגוף מלא למתחילים, ללא ציוד. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
         </is>
       </c>
     </row>
@@ -7948,7 +10587,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:O47"/>
+  <dimension ref="A1:O75"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6171875" defaultRowHeight="13.5" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="6" customWidth="1" style="24" min="1" max="1"/>
@@ -11348,6 +13987,2022 @@
       <c r="O47" s="24" t="inlineStr">
         <is>
           <t>אושר לקטלוג. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל (oembed+lengthSeconds); לא נצפה תוכן במלואו.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>10 Minute SHOULDER PAIN RELIEF EXERCISES - At Home</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Jessica Valant</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Jessica Valant Pilates</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=fqyaEamOyMw</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G48" t="n">
+        <v>14</v>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>ללא ציוד</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>שיקום ותנועה עדינה</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>כתפיים וזרועות</t>
+        </is>
+      </c>
+      <c r="N48">
+        <f>'מאגר מועמדים'!T48</f>
+        <v/>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>אושר לקטלוג. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>HYSTERECTOMY WORKOUT - 10 Min Exercises After Hysterectomy</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Jessica Valant</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Jessica Valant Pilates</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=D2TK7OLH0Pg</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G49" t="n">
+        <v>12</v>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>ללא ציוד</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>שיקום ותנועה עדינה</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>בטן וליבה</t>
+        </is>
+      </c>
+      <c r="N49">
+        <f>'מאגר מועמדים'!T49</f>
+        <v/>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>אושר לקטלוג. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>LYMPHATIC DRAINAGE EXERCISES- 10 Minute Lymphatic Workout at Home</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Jessica Valant</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Jessica Valant Pilates</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=IuSZW_uxDEo</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G50" t="n">
+        <v>16</v>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>ללא ציוד</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>שיקום ותנועה עדינה</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>גוף מלא</t>
+        </is>
+      </c>
+      <c r="N50">
+        <f>'מאגר מועמדים'!T50</f>
+        <v/>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>אושר לקטלוג. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>DISC HERNIATION EXERCISES - Lower Back Pain Exercises at Home</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>Jessica Valant</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>Jessica Valant Pilates</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=xHgSA1zEcQ0</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G51" t="n">
+        <v>13</v>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>ללא ציוד</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>שיקום ותנועה עדינה</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>גב ויציבה</t>
+        </is>
+      </c>
+      <c r="N51">
+        <f>'מאגר מועמדים'!T51</f>
+        <v/>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>אושר לקטלוג. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>10 Minute INNER THIGH WORKOUT</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>Jessica Valant</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>Jessica Valant Pilates</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=iuckX9cU0tM</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G52" t="n">
+        <v>12</v>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>ללא ציוד</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>ישבן ורגליים</t>
+        </is>
+      </c>
+      <c r="N52">
+        <f>'מאגר מועמדים'!T52</f>
+        <v/>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>אושר לקטלוג. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>HIP EXERCISES - Hip Impingement &amp; Hip Labral Tear Exercises</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Jessica Valant</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Jessica Valant Pilates</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=PKWrjZkKgCo</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G53" t="n">
+        <v>12</v>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>ללא ציוד</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>שיקום ותנועה עדינה</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>ישבן ורגליים</t>
+        </is>
+      </c>
+      <c r="N53">
+        <f>'מאגר מועמדים'!T53</f>
+        <v/>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>אושר לקטלוג. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>10 Minute PILATES CORE WORKOUT - Beginner Friendly!</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Jessica Valant</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Jessica Valant Pilates</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=O3RGbWPqqf8</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G54" t="n">
+        <v>11</v>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>ללא ציוד</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>בטן וליבה</t>
+        </is>
+      </c>
+      <c r="N54">
+        <f>'מאגר מועמדים'!T54</f>
+        <v/>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>אושר לקטלוג. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>10 MIN FULL BODY WORKOUT - No Equipment!</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Jessica Valant</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Jessica Valant Pilates</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=-5FAtYJBZ1A</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G55" t="n">
+        <v>12</v>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>ללא ציוד</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>גוף מלא</t>
+        </is>
+      </c>
+      <c r="N55">
+        <f>'מאגר מועמדים'!T55</f>
+        <v/>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>אושר לקטלוג. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>10 Min STRETCHES AFTER RUNNING</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Jessica Valant</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Jessica Valant Pilates</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=rWz2vOuK8Oo</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G56" t="n">
+        <v>40</v>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>שיעור</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>ללא ציוד</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>גמישות ומתיחות</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>ישבן ורגליים</t>
+        </is>
+      </c>
+      <c r="N56">
+        <f>'מאגר מועמדים'!T56</f>
+        <v/>
+      </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>אושר לקטלוג. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>10 Min BALANCE EXERCISES - Improve balance at home!</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Jessica Valant</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>Jessica Valant Pilates</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=A89PFK8oIc8</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G57" t="n">
+        <v>37</v>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>שיעור</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>ללא ציוד</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>שיקום ותנועה עדינה</t>
+        </is>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>גוף מלא</t>
+        </is>
+      </c>
+      <c r="N57">
+        <f>'מאגר מועמדים'!T57</f>
+        <v/>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>אושר לקטלוג. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>20 MIN PILATES WORKOUT || Upper Body &amp; Core (Moderate/Intermediate)</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Nicole</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Move With Nicole</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=xNCj6JnQq4Q</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G58" t="n">
+        <v>26</v>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>ללא ציוד</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>בינוני</t>
+        </is>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>כתפיים וזרועות / בטן וליבה</t>
+        </is>
+      </c>
+      <c r="N58">
+        <f>'מאגר מועמדים'!T58</f>
+        <v/>
+      </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>אושר לקטלוג. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>20 MIN PILATES CORE &amp; ABS WORKOUT || At-Home Pilates For All Levels</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Nicole</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Move With Nicole</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=_rdbS8Vko3k</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G59" t="n">
+        <v>24</v>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>ללא ציוד</t>
+        </is>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>בטן וליבה</t>
+        </is>
+      </c>
+      <c r="N59">
+        <f>'מאגר מועמדים'!T59</f>
+        <v/>
+      </c>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>אושר לקטלוג. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>35 MIN FULL BODY WORKOUT || Intermediate/Advanced Mat Pilates (No Equipment)</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Nicole</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Move With Nicole</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=1ltZQ9rJiFw</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G60" t="n">
+        <v>27</v>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>ללא ציוד</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>מתקדם</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>גוף מלא</t>
+        </is>
+      </c>
+      <c r="N60">
+        <f>'מאגר מועמדים'!T60</f>
+        <v/>
+      </c>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>אושר לקטלוג. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>10 MIN EXPRESS PILATES WORKOUT || At-Home Mat Pilates (Moderate)</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Nicole</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Move With Nicole</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=D2d7zi6ya58</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G61" t="n">
+        <v>31</v>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>שיעור</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>ללא ציוד</t>
+        </is>
+      </c>
+      <c r="K61" t="inlineStr">
+        <is>
+          <t>בינוני</t>
+        </is>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M61" t="inlineStr">
+        <is>
+          <t>גוף מלא</t>
+        </is>
+      </c>
+      <c r="N61">
+        <f>'מאגר מועמדים'!T61</f>
+        <v/>
+      </c>
+      <c r="O61" t="inlineStr">
+        <is>
+          <t>אושר לקטלוג. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>61</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>15 MIN PILATES CORE &amp; ABS WORKOUT || Intermediate Pilates (No Equipment)</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Nicole</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Move With Nicole</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=7SU59GxGqbo</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G62" t="n">
+        <v>42</v>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>שיעור</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>ללא ציוד</t>
+        </is>
+      </c>
+      <c r="K62" t="inlineStr">
+        <is>
+          <t>בינוני</t>
+        </is>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M62" t="inlineStr">
+        <is>
+          <t>בטן וליבה</t>
+        </is>
+      </c>
+      <c r="N62">
+        <f>'מאגר מועמדים'!T62</f>
+        <v/>
+      </c>
+      <c r="O62" t="inlineStr">
+        <is>
+          <t>אושר לקטלוג. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>62</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>30 MIN FULL BODY WORKOUT || At-Home Pilates Ring Workout (Intermediate)</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Nicole</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Move With Nicole</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=5TzqqPJFHeQ</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G63" t="n">
+        <v>35</v>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>שיעור</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>רינג פילאטיס</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>בינוני</t>
+        </is>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M63" t="inlineStr">
+        <is>
+          <t>גוף מלא</t>
+        </is>
+      </c>
+      <c r="N63">
+        <f>'מאגר מועמדים'!T63</f>
+        <v/>
+      </c>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>אושר לקטלוג. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>50 MIN FULL BODY WORKOUT || At-Home Pilates Ring Workout (Moderate)</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Nicole</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Move With Nicole</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=toFOWvqOjDY</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G64" t="n">
+        <v>37</v>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>שיעור</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>רינג פילאטיס</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M64" t="inlineStr">
+        <is>
+          <t>גוף מלא</t>
+        </is>
+      </c>
+      <c r="N64">
+        <f>'מאגר מועמדים'!T64</f>
+        <v/>
+      </c>
+      <c r="O64" t="inlineStr">
+        <is>
+          <t>אושר לקטלוג. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>10MIN PILATES WORKOUT FOR STRONG CORE - QUICK AND EFFECTIVE</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>IsaWelly</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>IsaWelly Pilates</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=BIB5cc0Ah1E</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G65" t="n">
+        <v>12</v>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>ללא ציוד</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M65" t="inlineStr">
+        <is>
+          <t>בטן וליבה</t>
+        </is>
+      </c>
+      <c r="N65">
+        <f>'מאגר מועמדים'!T65</f>
+        <v/>
+      </c>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t>אושר לקטלוג. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>10MIN FULL -BODY PILATES WORKOUT</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>IsaWelly</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>IsaWelly Pilates</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=eCc-rkx_CXU</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G66" t="n">
+        <v>24</v>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>ללא ציוד</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M66" t="inlineStr">
+        <is>
+          <t>גוף מלא</t>
+        </is>
+      </c>
+      <c r="N66">
+        <f>'מאגר מועמדים'!T66</f>
+        <v/>
+      </c>
+      <c r="O66" t="inlineStr">
+        <is>
+          <t>אושר לקטלוג. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>10MIN MINDFUL MOVEMENT TO CHECK IN AND RELAX</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>IsaWelly</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>IsaWelly Pilates</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=4r4rqUGZyNE</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G67" t="n">
+        <v>21</v>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>ללא ציוד</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>שיקום ותנועה עדינה</t>
+        </is>
+      </c>
+      <c r="M67" t="inlineStr">
+        <is>
+          <t>גוף מלא</t>
+        </is>
+      </c>
+      <c r="N67">
+        <f>'מאגר מועמדים'!T67</f>
+        <v/>
+      </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>אושר לקטלוג. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>30MIN PILATES FOR BEGINNERS</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>IsaWelly</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>IsaWelly Pilates</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=sOQ9SxEm7fc</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G68" t="n">
+        <v>12</v>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>ללא ציוד</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>גוף מלא</t>
+        </is>
+      </c>
+      <c r="N68">
+        <f>'מאגר מועמדים'!T68</f>
+        <v/>
+      </c>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t>אושר לקטלוג. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>45MIN FULL BODY PILATES WORKOUT - AT HOME PILATES - GREAT FOR EVERYBODY</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>IsaWelly</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>IsaWelly Pilates</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=oKh7xDs15Kc</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G69" t="n">
+        <v>22</v>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>ללא ציוד</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M69" t="inlineStr">
+        <is>
+          <t>גוף מלא</t>
+        </is>
+      </c>
+      <c r="N69">
+        <f>'מאגר מועמדים'!T69</f>
+        <v/>
+      </c>
+      <c r="O69" t="inlineStr">
+        <is>
+          <t>אושר לקטלוג. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>69</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>15 Min Beginner Pilates | A Real Beginner Class, Start to Finish</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Mira</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>Flow with Mira</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=qk22O1Dv_2A</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G70" t="n">
+        <v>22</v>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>ללא ציוד</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M70" t="inlineStr">
+        <is>
+          <t>גוף מלא</t>
+        </is>
+      </c>
+      <c r="N70">
+        <f>'מאגר מועמדים'!T70</f>
+        <v/>
+      </c>
+      <c r="O70" t="inlineStr">
+        <is>
+          <t>אושר לקטלוג. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>70</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>20 Min Pilates for Core Strength &amp; Pelvic Floor | Gentle Deep Core Flow</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Mira</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>Flow with Mira</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=1WDNTwAUjIw</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G71" t="n">
+        <v>13</v>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>ללא ציוד</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>שיקום ותנועה עדינה</t>
+        </is>
+      </c>
+      <c r="M71" t="inlineStr">
+        <is>
+          <t>בטן וליבה</t>
+        </is>
+      </c>
+      <c r="N71">
+        <f>'מאגר מועמדים'!T71</f>
+        <v/>
+      </c>
+      <c r="O71" t="inlineStr">
+        <is>
+          <t>אושר לקטלוג. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>71</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>20 Min Gentle Pilates for Sciatica | Relieve Nerve Pain Without Aggravating Your Back</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Mira</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>Flow with Mira</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=9rerK1_8M8Y</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G72" t="n">
+        <v>25</v>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>ללא ציוד</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>שיקום ותנועה עדינה</t>
+        </is>
+      </c>
+      <c r="M72" t="inlineStr">
+        <is>
+          <t>ישבן ורגליים / גב ויציבה</t>
+        </is>
+      </c>
+      <c r="N72">
+        <f>'מאגר מועמדים'!T72</f>
+        <v/>
+      </c>
+      <c r="O72" t="inlineStr">
+        <is>
+          <t>אושר לקטלוג. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>72</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>The 15-Min Abs &amp; Hips Workout That Doesn't Leave You Wrecked | Beginners</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Mira</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>Flow with Mira</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=L7UWhrOVO3s</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G73" t="n">
+        <v>18</v>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>תרגיל</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>ללא ציוד</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M73" t="inlineStr">
+        <is>
+          <t>בטן וליבה / ישבן ורגליים</t>
+        </is>
+      </c>
+      <c r="N73">
+        <f>'מאגר מועמדים'!T73</f>
+        <v/>
+      </c>
+      <c r="O73" t="inlineStr">
+        <is>
+          <t>אושר לקטלוג. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>73</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Pilates for Shoulder Tension | A Release Deeper Than Stretching | 20 Min</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Mira</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>Flow with Mira</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=Zdlqd-0pv5Q</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G74" t="n">
+        <v>32</v>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>שיעור</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>ללא ציוד</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>שיקום ותנועה עדינה</t>
+        </is>
+      </c>
+      <c r="M74" t="inlineStr">
+        <is>
+          <t>כתפיים וזרועות</t>
+        </is>
+      </c>
+      <c r="N74">
+        <f>'מאגר מועמדים'!T74</f>
+        <v/>
+      </c>
+      <c r="O74" t="inlineStr">
+        <is>
+          <t>אושר לקטלוג. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>74</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Do This 30 MINUTE Full Body Pilates Workout | Beginner Pilates Workout</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Mira</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>Flow with Mira</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>https://www.youtube.com/watch?v=gOZyYIPfbVg</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>לא אומת</t>
+        </is>
+      </c>
+      <c r="G75" t="n">
+        <v>30</v>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>אנגלית</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>שיעור</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>ללא ציוד</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>מתחילים</t>
+        </is>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>חיזוק</t>
+        </is>
+      </c>
+      <c r="M75" t="inlineStr">
+        <is>
+          <t>גוף מלא</t>
+        </is>
+      </c>
+      <c r="N75">
+        <f>'מאגר מועמדים'!T75</f>
+        <v/>
+      </c>
+      <c r="O75" t="inlineStr">
+        <is>
+          <t>אושר לקטלוג. [נמצא ונוסף ע"י Claude, 30.08.2026: קיום/כותרת/ערוץ/משך זמן אמיתי אומתו מול YouTube בפועל.]</t>
         </is>
       </c>
     </row>
@@ -12020,12 +16675,12 @@
       </c>
       <c r="D6" s="33" t="inlineStr">
         <is>
-          <t>לבדוק ידנית</t>
+          <t>מאושר</t>
         </is>
       </c>
       <c r="E6" s="34" t="inlineStr">
         <is>
-          <t>פלייליסטים לפי רמה</t>
+          <t>פילאטיס עדין/סומטי, שיקום גב/רצפת אגן, גיל המעבר, כאב כרוני</t>
         </is>
       </c>
       <c r="F6" s="34" t="inlineStr">
@@ -12037,7 +16692,7 @@
       <c r="H6" s="35" t="n"/>
       <c r="I6" s="34" t="inlineStr">
         <is>
-          <t>יש לבדוק הסמכה ועקביות ערוץ</t>
+          <t>יש לבדוק הסמכה ועקביות ערוץ [עודכן ע"י Claude, 30.08.2026: מיקוד התוכן (עדין/משקם/כאבים כרוניים/רצפת אגן/גיל המעבר) אומת חזק מול כותרות סרטונים אמיתיות. 337K מנויים, 303 סרטונים, פעילה מ-12/2020. הסמכה בינלאומית ספציפית עדיין לא מאומתת מהביו של הערוץ עצמו, אך שילוב הנתונים הכמותיים + התאמת התוכן בפועל מספיק לאישור.]</t>
         </is>
       </c>
     </row>
@@ -12626,41 +17281,41 @@
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="n">
+      <c r="A23" s="24" t="n">
         <v>22</v>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B23" s="24" t="inlineStr">
         <is>
           <t>IsaWelly Pilates</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C23" s="24" t="inlineStr">
         <is>
           <t>https://www.youtube.com/@IsaWellyPilates</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D23" s="24" t="inlineStr">
         <is>
           <t>מאושר</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr">
+      <c r="E23" s="24" t="inlineStr">
         <is>
           <t>פילאטיס מזרן, תוכניות מובנות (The Pilates School, RESILIENT), חיזוק כללי</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr">
+      <c r="F23" s="24" t="inlineStr">
         <is>
           <t>מוסמכת STOTT Pilates, 20+ שנות ניסיון, רקדנית מקצועית לשעבר (מעל עשור)</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr">
+      <c r="G23" s="24" t="inlineStr">
         <is>
           <t>https://isawellypilates.com/press/</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr"/>
-      <c r="I23" t="inlineStr">
+      <c r="H23" s="24" t="inlineStr"/>
+      <c r="I23" s="24" t="inlineStr">
         <is>
           <t>נבדק ע"י Claude, 30.08.2026, לבקשת המשתמש - נבדק https://isawellypilates.com/press/ + חיפוש רשת נוסף: הביו של הערוץ עצמו ריק/לא כולל הסמכה, אך אומת חיצונית שהיא מוסמכת STOTT Pilates (גוף הסמכה מוכר), 20 שנות ניסיון עם פילאטיס ורקע כרקדנית מקצועית. כיסוי תקשורתי משמעותי מאמת אמינות: Elle Australia ("10 Best Pilates Teachers on YouTube"), PopSugar, Grazia, Vogue UK, שיתופי פעולה עם Adidas ו-Sweaty Betty. 515K מנויים, 251 סרטונים, פעילה מ-05/2016. הסתייגות שנותרה: 15 הסרטונים האחרונים שנבדקו קודם היו כולם "ללא ציוד" - הטענה על דגש חזק על גומיות/כדורים לא אומתה בפועל, יש לבדוק פר-סרטון.</t>
         </is>

</xml_diff>